<commit_message>
Rhizosphere conductance estimation with respect to resistance percent up to water potential related stomatal closure
</commit_message>
<xml_diff>
--- a/data-raw/SpParamsMED.xlsx
+++ b/data-raw/SpParamsMED.xlsx
@@ -3674,7 +3674,9 @@
       <c r="AF2" t="n">
         <v>1.56</v>
       </c>
-      <c r="AG2"/>
+      <c r="AG2" t="n">
+        <v>0</v>
+      </c>
       <c r="AH2" t="n">
         <v>2.36476</v>
       </c>
@@ -4020,7 +4022,9 @@
       <c r="AF3" t="n">
         <v>1.56</v>
       </c>
-      <c r="AG3"/>
+      <c r="AG3" t="n">
+        <v>0</v>
+      </c>
       <c r="AH3" t="n">
         <v>2.36476</v>
       </c>
@@ -4592,7 +4596,9 @@
       <c r="AF5" t="n">
         <v>1.43</v>
       </c>
-      <c r="AG5"/>
+      <c r="AG5" t="n">
+        <v>0</v>
+      </c>
       <c r="AH5"/>
       <c r="AI5"/>
       <c r="AJ5"/>
@@ -6766,7 +6772,9 @@
       <c r="AF13" t="n">
         <v>1.7841</v>
       </c>
-      <c r="AG13"/>
+      <c r="AG13" t="n">
+        <v>0</v>
+      </c>
       <c r="AH13"/>
       <c r="AI13"/>
       <c r="AJ13"/>
@@ -11946,7 +11954,9 @@
       <c r="AF34" t="n">
         <v>1.7</v>
       </c>
-      <c r="AG34"/>
+      <c r="AG34" t="n">
+        <v>-0.041021302291958</v>
+      </c>
       <c r="AH34"/>
       <c r="AI34"/>
       <c r="AJ34"/>
@@ -12268,7 +12278,9 @@
       <c r="AF35" t="n">
         <v>1.56</v>
       </c>
-      <c r="AG35"/>
+      <c r="AG35" t="n">
+        <v>0</v>
+      </c>
       <c r="AH35" t="n">
         <v>2.36476</v>
       </c>
@@ -12772,9 +12784,15 @@
       <c r="AB37"/>
       <c r="AC37"/>
       <c r="AD37"/>
-      <c r="AE37"/>
-      <c r="AF37"/>
-      <c r="AG37"/>
+      <c r="AE37" t="n">
+        <v>0.118639640398548</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>1.62588</v>
+      </c>
+      <c r="AG37" t="n">
+        <v>0</v>
+      </c>
       <c r="AH37"/>
       <c r="AI37"/>
       <c r="AJ37"/>
@@ -26922,7 +26940,9 @@
       <c r="AF99" t="n">
         <v>1.7</v>
       </c>
-      <c r="AG99"/>
+      <c r="AG99" t="n">
+        <v>-0.0166666264109415</v>
+      </c>
       <c r="AH99" t="n">
         <v>3.85373</v>
       </c>
@@ -31622,9 +31642,15 @@
       <c r="AB118"/>
       <c r="AC118"/>
       <c r="AD118"/>
-      <c r="AE118"/>
-      <c r="AF118"/>
-      <c r="AG118"/>
+      <c r="AE118" t="n">
+        <v>0.230827770459304</v>
+      </c>
+      <c r="AF118" t="n">
+        <v>0.791981150129859</v>
+      </c>
+      <c r="AG118" t="n">
+        <v>0</v>
+      </c>
       <c r="AH118"/>
       <c r="AI118"/>
       <c r="AJ118"/>
@@ -32138,9 +32164,15 @@
       <c r="AB120"/>
       <c r="AC120"/>
       <c r="AD120"/>
-      <c r="AE120"/>
-      <c r="AF120"/>
-      <c r="AG120"/>
+      <c r="AE120" t="n">
+        <v>0.0875554428342399</v>
+      </c>
+      <c r="AF120" t="n">
+        <v>1.68286</v>
+      </c>
+      <c r="AG120" t="n">
+        <v>0</v>
+      </c>
       <c r="AH120"/>
       <c r="AI120"/>
       <c r="AJ120"/>
@@ -36262,9 +36294,15 @@
       <c r="AB137"/>
       <c r="AC137"/>
       <c r="AD137"/>
-      <c r="AE137"/>
-      <c r="AF137"/>
-      <c r="AG137"/>
+      <c r="AE137" t="n">
+        <v>0.0313703499974048</v>
+      </c>
+      <c r="AF137" t="n">
+        <v>1.53326</v>
+      </c>
+      <c r="AG137" t="n">
+        <v>0</v>
+      </c>
       <c r="AH137"/>
       <c r="AI137"/>
       <c r="AJ137"/>
@@ -38922,7 +38960,9 @@
       <c r="AF148" t="n">
         <v>1.56</v>
       </c>
-      <c r="AG148"/>
+      <c r="AG148" t="n">
+        <v>0</v>
+      </c>
       <c r="AH148" t="n">
         <v>2.36476</v>
       </c>
@@ -39472,9 +39512,15 @@
       <c r="AB150"/>
       <c r="AC150"/>
       <c r="AD150"/>
-      <c r="AE150"/>
-      <c r="AF150"/>
-      <c r="AG150"/>
+      <c r="AE150" t="n">
+        <v>0.0568488710473838</v>
+      </c>
+      <c r="AF150" t="n">
+        <v>1.52121763003559</v>
+      </c>
+      <c r="AG150" t="n">
+        <v>-0.0249465171770667</v>
+      </c>
       <c r="AH150"/>
       <c r="AI150"/>
       <c r="AJ150"/>
@@ -39800,7 +39846,9 @@
       <c r="AF151" t="n">
         <v>2.1014</v>
       </c>
-      <c r="AG151"/>
+      <c r="AG151" t="n">
+        <v>-0.028362858645325</v>
+      </c>
       <c r="AH151" t="n">
         <v>2.26205</v>
       </c>
@@ -40128,9 +40176,15 @@
       <c r="AB152"/>
       <c r="AC152"/>
       <c r="AD152"/>
-      <c r="AE152"/>
-      <c r="AF152"/>
-      <c r="AG152"/>
+      <c r="AE152" t="n">
+        <v>0.14306999757507</v>
+      </c>
+      <c r="AF152" t="n">
+        <v>1.36220507204865</v>
+      </c>
+      <c r="AG152" t="n">
+        <v>-0.0861234049842975</v>
+      </c>
       <c r="AH152"/>
       <c r="AI152"/>
       <c r="AJ152"/>
@@ -40424,9 +40478,15 @@
       <c r="AB153"/>
       <c r="AC153"/>
       <c r="AD153"/>
-      <c r="AE153"/>
-      <c r="AF153"/>
-      <c r="AG153"/>
+      <c r="AE153" t="n">
+        <v>0.039603626372559</v>
+      </c>
+      <c r="AF153" t="n">
+        <v>1.68688278125257</v>
+      </c>
+      <c r="AG153" t="n">
+        <v>-0.0672902010898818</v>
+      </c>
       <c r="AH153"/>
       <c r="AI153"/>
       <c r="AJ153"/>
@@ -40732,9 +40792,15 @@
       <c r="AB154"/>
       <c r="AC154"/>
       <c r="AD154"/>
-      <c r="AE154"/>
-      <c r="AF154"/>
-      <c r="AG154"/>
+      <c r="AE154" t="n">
+        <v>0.929364102112653</v>
+      </c>
+      <c r="AF154" t="n">
+        <v>0.753200986633843</v>
+      </c>
+      <c r="AG154" t="n">
+        <v>-0.0285867126524247</v>
+      </c>
       <c r="AH154"/>
       <c r="AI154"/>
       <c r="AJ154"/>
@@ -41018,7 +41084,9 @@
       <c r="AF155" t="n">
         <v>2.1826</v>
       </c>
-      <c r="AG155"/>
+      <c r="AG155" t="n">
+        <v>-0.0387677691224012</v>
+      </c>
       <c r="AH155" t="n">
         <v>1.50576</v>
       </c>
@@ -41358,9 +41426,15 @@
       <c r="AB156"/>
       <c r="AC156"/>
       <c r="AD156"/>
-      <c r="AE156"/>
-      <c r="AF156"/>
-      <c r="AG156"/>
+      <c r="AE156" t="n">
+        <v>0.173868488462801</v>
+      </c>
+      <c r="AF156" t="n">
+        <v>1.23647203497902</v>
+      </c>
+      <c r="AG156" t="n">
+        <v>-0.0166378429635153</v>
+      </c>
       <c r="AH156"/>
       <c r="AI156"/>
       <c r="AJ156"/>
@@ -43524,7 +43598,9 @@
       <c r="AF164" t="n">
         <v>1.56</v>
       </c>
-      <c r="AG164"/>
+      <c r="AG164" t="n">
+        <v>0</v>
+      </c>
       <c r="AH164" t="n">
         <v>2.36476</v>
       </c>
@@ -44108,9 +44184,15 @@
       <c r="AB166"/>
       <c r="AC166"/>
       <c r="AD166"/>
-      <c r="AE166"/>
-      <c r="AF166"/>
-      <c r="AG166"/>
+      <c r="AE166" t="n">
+        <v>0.106305422918705</v>
+      </c>
+      <c r="AF166" t="n">
+        <v>1.321636004093</v>
+      </c>
+      <c r="AG166" t="n">
+        <v>0</v>
+      </c>
       <c r="AH166"/>
       <c r="AI166"/>
       <c r="AJ166"/>
@@ -44638,9 +44720,15 @@
       <c r="AB168"/>
       <c r="AC168"/>
       <c r="AD168"/>
-      <c r="AE168"/>
-      <c r="AF168"/>
-      <c r="AG168"/>
+      <c r="AE168" t="n">
+        <v>0.0196870235378835</v>
+      </c>
+      <c r="AF168" t="n">
+        <v>1.96752</v>
+      </c>
+      <c r="AG168" t="n">
+        <v>0</v>
+      </c>
       <c r="AH168"/>
       <c r="AI168"/>
       <c r="AJ168"/>
@@ -45182,9 +45270,15 @@
       </c>
       <c r="AC170"/>
       <c r="AD170"/>
-      <c r="AE170"/>
-      <c r="AF170"/>
-      <c r="AG170"/>
+      <c r="AE170" t="n">
+        <v>0.0631063048187397</v>
+      </c>
+      <c r="AF170" t="n">
+        <v>1.54503172767883</v>
+      </c>
+      <c r="AG170" t="n">
+        <v>-0.00528847613004736</v>
+      </c>
       <c r="AH170"/>
       <c r="AI170"/>
       <c r="AJ170"/>
@@ -45750,7 +45844,9 @@
       <c r="AF172" t="n">
         <v>1.7</v>
       </c>
-      <c r="AG172"/>
+      <c r="AG172" t="n">
+        <v>-0.0329883123011257</v>
+      </c>
       <c r="AH172"/>
       <c r="AI172"/>
       <c r="AJ172"/>
@@ -46662,7 +46758,9 @@
       <c r="AF175" t="n">
         <v>1.7</v>
       </c>
-      <c r="AG175"/>
+      <c r="AG175" t="n">
+        <v>0</v>
+      </c>
       <c r="AH175"/>
       <c r="AI175"/>
       <c r="AJ175"/>
@@ -47268,9 +47366,15 @@
       <c r="AB177"/>
       <c r="AC177"/>
       <c r="AD177"/>
-      <c r="AE177"/>
-      <c r="AF177"/>
-      <c r="AG177"/>
+      <c r="AE177" t="n">
+        <v>0.032248314976163</v>
+      </c>
+      <c r="AF177" t="n">
+        <v>1.36447502453626</v>
+      </c>
+      <c r="AG177" t="n">
+        <v>-0.00987413307430693</v>
+      </c>
       <c r="AH177"/>
       <c r="AI177"/>
       <c r="AJ177"/>
@@ -53354,7 +53458,9 @@
       <c r="AF202" t="n">
         <v>1.56</v>
       </c>
-      <c r="AG202"/>
+      <c r="AG202" t="n">
+        <v>0</v>
+      </c>
       <c r="AH202" t="n">
         <v>2.36476</v>
       </c>

</xml_diff>

<commit_message>
update SpParams and other
</commit_message>
<xml_diff>
--- a/data-raw/SpParamsMED.xlsx
+++ b/data-raw/SpParamsMED.xlsx
@@ -3674,7 +3674,7 @@
         <v>2500</v>
       </c>
       <c r="Q2" t="n">
-        <v>7738.00000000001</v>
+        <v>2938.63837507692</v>
       </c>
       <c r="R2" t="n">
         <v>200</v>
@@ -3833,7 +3833,7 @@
         <v>120.634920634921</v>
       </c>
       <c r="DB2" t="n">
-        <v>0.0004035</v>
+        <v>0.6</v>
       </c>
       <c r="DC2" t="n">
         <v>-3.1</v>
@@ -3847,12 +3847,14 @@
       <c r="DF2" t="n">
         <v>80</v>
       </c>
-      <c r="DG2"/>
+      <c r="DG2" t="n">
+        <v>0.368914872</v>
+      </c>
       <c r="DH2" t="n">
         <v>-0.53</v>
       </c>
       <c r="DI2" t="n">
-        <v>-3.14</v>
+        <v>-3.3</v>
       </c>
       <c r="DJ2" t="n">
         <v>-4.39</v>
@@ -3975,7 +3977,7 @@
         <v>170</v>
       </c>
       <c r="P3" t="n">
-        <v>1570</v>
+        <v>1690</v>
       </c>
       <c r="Q3" t="n">
         <v>3300</v>
@@ -4001,9 +4003,15 @@
       <c r="AB3"/>
       <c r="AC3"/>
       <c r="AD3"/>
-      <c r="AE3"/>
-      <c r="AF3"/>
-      <c r="AG3"/>
+      <c r="AE3" t="n">
+        <v>0.170586159355792</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>1.37822466400964</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>0.00214453867981628</v>
+      </c>
       <c r="AH3" t="n">
         <v>2.36476</v>
       </c>
@@ -4028,8 +4036,12 @@
       <c r="AO3" t="n">
         <v>0.538</v>
       </c>
-      <c r="AP3"/>
-      <c r="AQ3"/>
+      <c r="AP3" t="n">
+        <v>0.667239487171173</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>0.817502081394196</v>
+      </c>
       <c r="AR3" t="n">
         <v>8.14364350796509</v>
       </c>
@@ -4065,7 +4077,7 @@
       </c>
       <c r="BG3"/>
       <c r="BH3" t="n">
-        <v>17000</v>
+        <v>17006.8027210884</v>
       </c>
       <c r="BI3"/>
       <c r="BJ3"/>
@@ -4141,7 +4153,7 @@
       <c r="CZ3"/>
       <c r="DA3"/>
       <c r="DB3" t="n">
-        <v>1.299505</v>
+        <v>0.88</v>
       </c>
       <c r="DC3" t="n">
         <v>-3.02</v>
@@ -4289,10 +4301,10 @@
         <v>170</v>
       </c>
       <c r="P4" t="n">
-        <v>1170</v>
+        <v>1230</v>
       </c>
       <c r="Q4" t="n">
-        <v>2548</v>
+        <v>2558</v>
       </c>
       <c r="R4" t="n">
         <v>150</v>
@@ -4315,19 +4327,45 @@
       <c r="AB4"/>
       <c r="AC4"/>
       <c r="AD4"/>
-      <c r="AE4"/>
-      <c r="AF4"/>
-      <c r="AG4"/>
-      <c r="AH4"/>
-      <c r="AI4"/>
-      <c r="AJ4"/>
-      <c r="AK4"/>
-      <c r="AL4"/>
-      <c r="AM4"/>
-      <c r="AN4"/>
-      <c r="AO4"/>
-      <c r="AP4"/>
-      <c r="AQ4"/>
+      <c r="AE4" t="n">
+        <v>0.170586159355792</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>1.37822466400964</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0.00214453867981628</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>2.36476</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>-0.763</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>-0.02285</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0.000074049</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>-0.01018</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>-0.27004</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>1.09636482208082</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>0.538</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>0.667239487171173</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>0.817502081394196</v>
+      </c>
       <c r="AR4"/>
       <c r="AS4"/>
       <c r="AT4"/>
@@ -4537,10 +4575,10 @@
         <v>183</v>
       </c>
       <c r="P5" t="n">
-        <v>1280</v>
+        <v>1000</v>
       </c>
       <c r="Q5" t="n">
-        <v>2691</v>
+        <v>2550</v>
       </c>
       <c r="R5"/>
       <c r="S5"/>
@@ -4548,10 +4586,10 @@
         <v>6962.5</v>
       </c>
       <c r="U5" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="V5" t="n">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="W5"/>
       <c r="X5"/>
@@ -4838,7 +4876,7 @@
         <v>700</v>
       </c>
       <c r="Q6" t="n">
-        <v>3500</v>
+        <v>2049.15433718182</v>
       </c>
       <c r="R6" t="n">
         <v>80</v>
@@ -4919,7 +4957,7 @@
       </c>
       <c r="BG6"/>
       <c r="BH6" t="n">
-        <v>7365</v>
+        <v>6802.72108843537</v>
       </c>
       <c r="BI6"/>
       <c r="BJ6" t="n">
@@ -5003,7 +5041,7 @@
         <v>69.7247706422018</v>
       </c>
       <c r="DB6" t="n">
-        <v>1.42</v>
+        <v>0.64</v>
       </c>
       <c r="DC6" t="n">
         <v>-3.83</v>
@@ -5015,7 +5053,9 @@
       <c r="DF6" t="n">
         <v>77</v>
       </c>
-      <c r="DG6"/>
+      <c r="DG6" t="n">
+        <v>1.223272505</v>
+      </c>
       <c r="DH6" t="n">
         <v>-0.82</v>
       </c>
@@ -5147,10 +5187,10 @@
         <v>183</v>
       </c>
       <c r="P7" t="n">
-        <v>400</v>
+        <v>870</v>
       </c>
       <c r="Q7" t="n">
-        <v>1941</v>
+        <v>2050</v>
       </c>
       <c r="R7"/>
       <c r="S7"/>
@@ -5293,7 +5333,7 @@
       <c r="CZ7"/>
       <c r="DA7"/>
       <c r="DB7" t="n">
-        <v>0.4348677</v>
+        <v>0.43</v>
       </c>
       <c r="DC7" t="n">
         <v>-4.87</v>
@@ -5441,10 +5481,10 @@
         <v>170</v>
       </c>
       <c r="P8" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="Q8" t="n">
-        <v>1350</v>
+        <v>1448</v>
       </c>
       <c r="R8"/>
       <c r="S8"/>
@@ -5509,7 +5549,7 @@
       </c>
       <c r="BG8"/>
       <c r="BH8" t="n">
-        <v>3400</v>
+        <v>3404.91601774642</v>
       </c>
       <c r="BI8"/>
       <c r="BJ8" t="n">
@@ -5577,7 +5617,7 @@
       <c r="CZ8"/>
       <c r="DA8"/>
       <c r="DB8" t="n">
-        <v>1.76</v>
+        <v>0.703842936</v>
       </c>
       <c r="DC8" t="n">
         <v>-5.73</v>
@@ -5589,7 +5629,9 @@
       <c r="DF8" t="n">
         <v>49.6</v>
       </c>
-      <c r="DG8"/>
+      <c r="DG8" t="n">
+        <v>1.223272505</v>
+      </c>
       <c r="DH8" t="n">
         <v>-0.86216</v>
       </c>
@@ -5725,10 +5767,10 @@
         <v>170</v>
       </c>
       <c r="P9" t="n">
-        <v>400</v>
+        <v>770</v>
       </c>
       <c r="Q9" t="n">
-        <v>1764</v>
+        <v>1781</v>
       </c>
       <c r="R9" t="n">
         <v>100</v>
@@ -5861,7 +5903,7 @@
       <c r="CZ9"/>
       <c r="DA9"/>
       <c r="DB9" t="n">
-        <v>17.04</v>
+        <v>1.32</v>
       </c>
       <c r="DC9" t="n">
         <v>-1.56</v>
@@ -6003,10 +6045,10 @@
         <v>170</v>
       </c>
       <c r="P10" t="n">
-        <v>100</v>
+        <v>690</v>
       </c>
       <c r="Q10" t="n">
-        <v>1850</v>
+        <v>2100</v>
       </c>
       <c r="R10"/>
       <c r="S10"/>
@@ -6261,10 +6303,10 @@
         <v>170</v>
       </c>
       <c r="P11" t="n">
-        <v>500</v>
+        <v>1150</v>
       </c>
       <c r="Q11" t="n">
-        <v>2835</v>
+        <v>3038</v>
       </c>
       <c r="R11" t="n">
         <v>150</v>
@@ -6395,7 +6437,7 @@
       <c r="CZ11"/>
       <c r="DA11"/>
       <c r="DB11" t="n">
-        <v>1</v>
+        <v>0.45</v>
       </c>
       <c r="DC11" t="n">
         <v>-3.68</v>
@@ -6533,10 +6575,10 @@
         <v>190</v>
       </c>
       <c r="P12" t="n">
-        <v>450</v>
+        <v>1000</v>
       </c>
       <c r="Q12" t="n">
-        <v>2384</v>
+        <v>2400</v>
       </c>
       <c r="R12" t="n">
         <v>80</v>
@@ -6546,10 +6588,10 @@
         <v>2090.625</v>
       </c>
       <c r="U12" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="V12" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="W12"/>
       <c r="X12"/>
@@ -6687,7 +6729,7 @@
       </c>
       <c r="DA12"/>
       <c r="DB12" t="n">
-        <v>0.866666666666667</v>
+        <v>0.38</v>
       </c>
       <c r="DC12" t="n">
         <v>-2.64</v>
@@ -7059,10 +7101,10 @@
         <v>170</v>
       </c>
       <c r="P14" t="n">
-        <v>700</v>
+        <v>900</v>
       </c>
       <c r="Q14" t="n">
-        <v>1821</v>
+        <v>1880</v>
       </c>
       <c r="R14" t="n">
         <v>100</v>
@@ -7072,10 +7114,10 @@
         <v>713.128163222</v>
       </c>
       <c r="U14" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="V14" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="W14"/>
       <c r="X14"/>
@@ -7325,10 +7367,10 @@
         <v>190</v>
       </c>
       <c r="P15" t="n">
-        <v>1450</v>
+        <v>1500</v>
       </c>
       <c r="Q15" t="n">
-        <v>2600</v>
+        <v>2650</v>
       </c>
       <c r="R15"/>
       <c r="S15"/>
@@ -7336,10 +7378,10 @@
         <v>387.58</v>
       </c>
       <c r="U15" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="V15" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="W15"/>
       <c r="X15"/>
@@ -7454,14 +7496,12 @@
       <c r="CY15"/>
       <c r="CZ15"/>
       <c r="DA15"/>
-      <c r="DB15" t="n">
-        <v>0.0000479</v>
-      </c>
+      <c r="DB15"/>
       <c r="DC15" t="n">
         <v>-1.5</v>
       </c>
       <c r="DD15" t="n">
-        <v>-2.2</v>
+        <v>-1.6</v>
       </c>
       <c r="DE15" t="n">
         <v>-2.3</v>
@@ -7615,7 +7655,7 @@
         <v>183</v>
       </c>
       <c r="P16" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q16" t="n">
         <v>400</v>
@@ -8055,10 +8095,10 @@
         <v>190</v>
       </c>
       <c r="P18" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="Q18" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="R18"/>
       <c r="S18"/>
@@ -8713,10 +8753,10 @@
         <v>183</v>
       </c>
       <c r="P21" t="n">
-        <v>450</v>
+        <v>700</v>
       </c>
       <c r="Q21" t="n">
-        <v>1788</v>
+        <v>1852</v>
       </c>
       <c r="R21"/>
       <c r="S21"/>
@@ -8922,7 +8962,7 @@
         <v>300</v>
       </c>
       <c r="Q22" t="n">
-        <v>1380.744</v>
+        <v>1734.9301185</v>
       </c>
       <c r="R22" t="n">
         <v>129.7478182</v>
@@ -8985,7 +9025,7 @@
         <v>0.0184942321007697</v>
       </c>
       <c r="BH22" t="n">
-        <v>1990</v>
+        <v>1993.08002614921</v>
       </c>
       <c r="BI22"/>
       <c r="BJ22" t="n">
@@ -9071,7 +9111,7 @@
         <v>32.9004329004329</v>
       </c>
       <c r="DB22" t="n">
-        <v>2.06</v>
+        <v>0.531</v>
       </c>
       <c r="DC22" t="n">
         <v>-6.93</v>
@@ -9080,12 +9120,14 @@
         <v>-7.84</v>
       </c>
       <c r="DE22" t="n">
-        <v>-9.77004985</v>
+        <v>-8.5</v>
       </c>
       <c r="DF22" t="n">
-        <v>26.7600936652573</v>
-      </c>
-      <c r="DG22"/>
+        <v>48.4076433121019</v>
+      </c>
+      <c r="DG22" t="n">
+        <v>1.589581219</v>
+      </c>
       <c r="DH22" t="n">
         <v>-0.20761</v>
       </c>
@@ -9209,10 +9251,10 @@
         <v>183</v>
       </c>
       <c r="P23" t="n">
-        <v>525</v>
+        <v>700</v>
       </c>
       <c r="Q23" t="n">
-        <v>1132</v>
+        <v>1146</v>
       </c>
       <c r="R23"/>
       <c r="S23"/>
@@ -9427,10 +9469,10 @@
         <v>183</v>
       </c>
       <c r="P24" t="n">
-        <v>100</v>
+        <v>350</v>
       </c>
       <c r="Q24" t="n">
-        <v>920</v>
+        <v>1000</v>
       </c>
       <c r="R24"/>
       <c r="S24"/>
@@ -9517,7 +9559,7 @@
         <v>0.0184942321007697</v>
       </c>
       <c r="BH24" t="n">
-        <v>1990</v>
+        <v>1993.08002614921</v>
       </c>
       <c r="BI24"/>
       <c r="BJ24" t="n">
@@ -9610,12 +9652,14 @@
         <v>-7.84</v>
       </c>
       <c r="DE24" t="n">
-        <v>-9.77004985</v>
+        <v>-8.5</v>
       </c>
       <c r="DF24" t="n">
-        <v>26.7600936652573</v>
-      </c>
-      <c r="DG24"/>
+        <v>48.4076433121019</v>
+      </c>
+      <c r="DG24" t="n">
+        <v>1.589581219</v>
+      </c>
       <c r="DH24" t="n">
         <v>-0.20761</v>
       </c>
@@ -10085,7 +10129,7 @@
       <c r="BF26"/>
       <c r="BG26"/>
       <c r="BH26" t="n">
-        <v>4530</v>
+        <v>4304.68565033038</v>
       </c>
       <c r="BI26"/>
       <c r="BJ26" t="n">
@@ -10153,13 +10197,13 @@
       <c r="CZ26"/>
       <c r="DA26"/>
       <c r="DB26" t="n">
-        <v>0.708</v>
+        <v>0.9</v>
       </c>
       <c r="DC26" t="n">
         <v>-2.17614</v>
       </c>
       <c r="DD26" t="n">
-        <v>-2.8</v>
+        <v>-3</v>
       </c>
       <c r="DE26" t="n">
         <v>-4.91662</v>
@@ -11243,10 +11287,10 @@
         <v>190</v>
       </c>
       <c r="P31" t="n">
-        <v>900</v>
+        <v>1150</v>
       </c>
       <c r="Q31" t="n">
-        <v>2215</v>
+        <v>2250</v>
       </c>
       <c r="R31" t="n">
         <v>76.2</v>
@@ -11256,10 +11300,10 @@
         <v>1000</v>
       </c>
       <c r="U31" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="V31" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="W31"/>
       <c r="X31"/>
@@ -11317,7 +11361,7 @@
       </c>
       <c r="BG31"/>
       <c r="BH31" t="n">
-        <v>4770</v>
+        <v>5347.5935828877</v>
       </c>
       <c r="BI31"/>
       <c r="BJ31" t="n">
@@ -11386,12 +11430,12 @@
       </c>
       <c r="CX31"/>
       <c r="CY31" t="n">
-        <v>-3.37</v>
+        <v>-1.77</v>
       </c>
       <c r="CZ31"/>
       <c r="DA31"/>
       <c r="DB31" t="n">
-        <v>3.62</v>
+        <v>3.07</v>
       </c>
       <c r="DC31" t="n">
         <v>-1.7</v>
@@ -11557,10 +11601,10 @@
         <v>190</v>
       </c>
       <c r="P32" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="Q32" t="n">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="R32"/>
       <c r="S32"/>
@@ -11786,7 +11830,7 @@
         <v>250</v>
       </c>
       <c r="Q33" t="n">
-        <v>1600</v>
+        <v>500</v>
       </c>
       <c r="R33"/>
       <c r="S33"/>
@@ -12035,10 +12079,10 @@
         <v>190</v>
       </c>
       <c r="P34" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q34" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="R34"/>
       <c r="S34"/>
@@ -12321,10 +12365,10 @@
         <v>190</v>
       </c>
       <c r="P35" t="n">
-        <v>300</v>
+        <v>70</v>
       </c>
       <c r="Q35" t="n">
-        <v>300</v>
+        <v>244</v>
       </c>
       <c r="R35"/>
       <c r="S35"/>
@@ -12344,30 +12388,14 @@
       <c r="AE35"/>
       <c r="AF35"/>
       <c r="AG35"/>
-      <c r="AH35" t="n">
-        <v>2.36476</v>
-      </c>
-      <c r="AI35" t="n">
-        <v>-0.763</v>
-      </c>
-      <c r="AJ35" t="n">
-        <v>-0.02285</v>
-      </c>
-      <c r="AK35" t="n">
-        <v>0.000074049</v>
-      </c>
-      <c r="AL35" t="n">
-        <v>-0.01018</v>
-      </c>
-      <c r="AM35" t="n">
-        <v>-0.27004</v>
-      </c>
-      <c r="AN35" t="n">
-        <v>1.09636482208082</v>
-      </c>
-      <c r="AO35" t="n">
-        <v>0.538</v>
-      </c>
+      <c r="AH35"/>
+      <c r="AI35"/>
+      <c r="AJ35"/>
+      <c r="AK35"/>
+      <c r="AL35"/>
+      <c r="AM35"/>
+      <c r="AN35"/>
+      <c r="AO35"/>
       <c r="AP35"/>
       <c r="AQ35"/>
       <c r="AR35"/>
@@ -12820,7 +12848,7 @@
         <v>2500</v>
       </c>
       <c r="Q37" t="n">
-        <v>3000</v>
+        <v>2578.089726</v>
       </c>
       <c r="R37" t="n">
         <v>89.0553191489362</v>
@@ -12945,7 +12973,7 @@
       <c r="CZ37"/>
       <c r="DA37"/>
       <c r="DB37" t="n">
-        <v>0.6250094</v>
+        <v>1.25</v>
       </c>
       <c r="DC37" t="n">
         <v>-3.16</v>
@@ -13073,10 +13101,10 @@
         <v>190</v>
       </c>
       <c r="P38" t="n">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="Q38" t="n">
-        <v>2250</v>
+        <v>2300</v>
       </c>
       <c r="R38" t="n">
         <v>200</v>
@@ -13373,10 +13401,10 @@
         <v>170</v>
       </c>
       <c r="P39" t="n">
-        <v>4000</v>
+        <v>1325</v>
       </c>
       <c r="Q39" t="n">
-        <v>7500</v>
+        <v>2875</v>
       </c>
       <c r="R39" t="n">
         <v>200</v>
@@ -13385,8 +13413,12 @@
       <c r="T39" t="n">
         <v>2400</v>
       </c>
-      <c r="U39"/>
-      <c r="V39"/>
+      <c r="U39" t="n">
+        <v>43</v>
+      </c>
+      <c r="V39" t="n">
+        <v>100</v>
+      </c>
       <c r="W39"/>
       <c r="X39"/>
       <c r="Y39"/>
@@ -13395,19 +13427,45 @@
       <c r="AB39"/>
       <c r="AC39"/>
       <c r="AD39"/>
-      <c r="AE39"/>
-      <c r="AF39"/>
-      <c r="AG39"/>
-      <c r="AH39"/>
-      <c r="AI39"/>
-      <c r="AJ39"/>
-      <c r="AK39"/>
-      <c r="AL39"/>
-      <c r="AM39"/>
-      <c r="AN39"/>
-      <c r="AO39"/>
-      <c r="AP39"/>
-      <c r="AQ39"/>
+      <c r="AE39" t="n">
+        <v>0.170586159355792</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>1.37822466400964</v>
+      </c>
+      <c r="AG39" t="n">
+        <v>0.00214453867981628</v>
+      </c>
+      <c r="AH39" t="n">
+        <v>2.36476</v>
+      </c>
+      <c r="AI39" t="n">
+        <v>-0.763</v>
+      </c>
+      <c r="AJ39" t="n">
+        <v>-0.02285</v>
+      </c>
+      <c r="AK39" t="n">
+        <v>0.000074049</v>
+      </c>
+      <c r="AL39" t="n">
+        <v>-0.01018</v>
+      </c>
+      <c r="AM39" t="n">
+        <v>-0.27004</v>
+      </c>
+      <c r="AN39" t="n">
+        <v>1.09636482208082</v>
+      </c>
+      <c r="AO39" t="n">
+        <v>0.538</v>
+      </c>
+      <c r="AP39" t="n">
+        <v>0.667239487171173</v>
+      </c>
+      <c r="AQ39" t="n">
+        <v>0.817502081394196</v>
+      </c>
       <c r="AR39"/>
       <c r="AS39"/>
       <c r="AT39"/>
@@ -13487,7 +13545,7 @@
       <c r="CZ39"/>
       <c r="DA39"/>
       <c r="DB39" t="n">
-        <v>0.0006702</v>
+        <v>0.37</v>
       </c>
       <c r="DC39" t="n">
         <v>-4.45</v>
@@ -13497,7 +13555,7 @@
       </c>
       <c r="DE39"/>
       <c r="DF39" t="n">
-        <v>16.78</v>
+        <v>22</v>
       </c>
       <c r="DG39"/>
       <c r="DH39" t="n">
@@ -13617,10 +13675,10 @@
         <v>190</v>
       </c>
       <c r="P40" t="n">
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="Q40" t="n">
-        <v>1967</v>
+        <v>1789</v>
       </c>
       <c r="R40"/>
       <c r="S40"/>
@@ -13857,10 +13915,10 @@
         <v>183</v>
       </c>
       <c r="P41" t="n">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="Q41" t="n">
-        <v>1000</v>
+        <v>1032</v>
       </c>
       <c r="R41"/>
       <c r="S41"/>
@@ -13987,7 +14045,7 @@
       <c r="CZ41"/>
       <c r="DA41"/>
       <c r="DB41" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="DC41" t="n">
         <v>-7.2</v>
@@ -14131,10 +14189,10 @@
         <v>170</v>
       </c>
       <c r="P42" t="n">
-        <v>1600</v>
+        <v>1650</v>
       </c>
       <c r="Q42" t="n">
-        <v>2476</v>
+        <v>2480</v>
       </c>
       <c r="R42"/>
       <c r="S42"/>
@@ -14235,7 +14293,7 @@
       <c r="CZ42"/>
       <c r="DA42"/>
       <c r="DB42" t="n">
-        <v>0.0004298</v>
+        <v>0.150259</v>
       </c>
       <c r="DC42"/>
       <c r="DD42" t="n">
@@ -14567,10 +14625,10 @@
         <v>183</v>
       </c>
       <c r="P44" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q44" t="n">
-        <v>100</v>
+        <v>267</v>
       </c>
       <c r="R44"/>
       <c r="S44"/>
@@ -14787,10 +14845,10 @@
         <v>190</v>
       </c>
       <c r="P45" t="n">
-        <v>196.081081081081</v>
+        <v>50</v>
       </c>
       <c r="Q45" t="n">
-        <v>422.378378378378</v>
+        <v>150</v>
       </c>
       <c r="R45"/>
       <c r="S45"/>
@@ -14987,10 +15045,10 @@
         <v>190</v>
       </c>
       <c r="P46" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="Q46" t="n">
-        <v>200</v>
+        <v>187.531172069825</v>
       </c>
       <c r="R46"/>
       <c r="S46"/>
@@ -15051,7 +15109,7 @@
         <v>0.136</v>
       </c>
       <c r="BH46" t="n">
-        <v>1460</v>
+        <v>1457.72594752187</v>
       </c>
       <c r="BI46"/>
       <c r="BJ46" t="n">
@@ -15121,21 +15179,21 @@
       <c r="CZ46"/>
       <c r="DA46"/>
       <c r="DB46" t="n">
-        <v>1.05</v>
+        <v>0.652</v>
       </c>
       <c r="DC46" t="n">
-        <v>-8.3</v>
+        <v>-7.2</v>
       </c>
       <c r="DD46" t="n">
         <v>-10.2</v>
       </c>
-      <c r="DE46" t="n">
-        <v>-13.5612816175</v>
-      </c>
+      <c r="DE46"/>
       <c r="DF46" t="n">
-        <v>14.4451495900181</v>
-      </c>
-      <c r="DG46"/>
+        <v>20.5405405405405</v>
+      </c>
+      <c r="DG46" t="n">
+        <v>1.461656823</v>
+      </c>
       <c r="DH46" t="n">
         <v>-0.8154</v>
       </c>
@@ -15254,7 +15312,7 @@
         <v>50</v>
       </c>
       <c r="Q47" t="n">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="R47"/>
       <c r="S47"/>
@@ -15325,7 +15383,7 @@
         <v>0.16</v>
       </c>
       <c r="BH47" t="n">
-        <v>3530</v>
+        <v>3527.22488527701</v>
       </c>
       <c r="BI47"/>
       <c r="BJ47" t="n">
@@ -15395,17 +15453,21 @@
       <c r="DB47" t="n">
         <v>0.170859771</v>
       </c>
-      <c r="DC47"/>
+      <c r="DC47" t="n">
+        <v>-2.7013</v>
+      </c>
       <c r="DD47" t="n">
         <v>-5.78</v>
       </c>
       <c r="DE47" t="n">
-        <v>-13.5612816175</v>
+        <v>-8.8587</v>
       </c>
       <c r="DF47" t="n">
-        <v>15.849100065125</v>
-      </c>
-      <c r="DG47"/>
+        <v>12.3428719914249</v>
+      </c>
+      <c r="DG47" t="n">
+        <v>1.461656823</v>
+      </c>
       <c r="DH47" t="n">
         <v>-0.8154</v>
       </c>
@@ -15758,7 +15820,7 @@
         <v>100</v>
       </c>
       <c r="Q49" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="R49"/>
       <c r="S49"/>
@@ -16251,7 +16313,7 @@
         <v>0.139</v>
       </c>
       <c r="BH51" t="n">
-        <v>1460</v>
+        <v>1457.72594752187</v>
       </c>
       <c r="BI51"/>
       <c r="BJ51" t="n">
@@ -16313,17 +16375,19 @@
       <c r="CZ51"/>
       <c r="DA51"/>
       <c r="DB51" t="n">
-        <v>0.716</v>
-      </c>
-      <c r="DC51"/>
+        <v>0.652</v>
+      </c>
+      <c r="DC51" t="n">
+        <v>-7.9</v>
+      </c>
       <c r="DD51" t="n">
-        <v>-6.2</v>
+        <v>-8.9</v>
       </c>
       <c r="DE51" t="n">
         <v>-11.18</v>
       </c>
       <c r="DF51" t="n">
-        <v>7.63052208835341</v>
+        <v>23.1707317073171</v>
       </c>
       <c r="DG51"/>
       <c r="DH51"/>
@@ -16505,7 +16569,7 @@
         <v>0.067326043135517</v>
       </c>
       <c r="BH52" t="n">
-        <v>1400</v>
+        <v>1403.18185517479</v>
       </c>
       <c r="BI52"/>
       <c r="BJ52" t="n">
@@ -16563,7 +16627,7 @@
       <c r="CZ52"/>
       <c r="DA52"/>
       <c r="DB52" t="n">
-        <v>0.5025626</v>
+        <v>0.502562594</v>
       </c>
       <c r="DC52" t="n">
         <v>-0.94335</v>
@@ -16577,7 +16641,9 @@
       <c r="DF52" t="n">
         <v>14.0394953170894</v>
       </c>
-      <c r="DG52"/>
+      <c r="DG52" t="n">
+        <v>2.5350134</v>
+      </c>
       <c r="DH52" t="n">
         <v>-0.01735</v>
       </c>
@@ -17393,10 +17459,10 @@
         <v>190</v>
       </c>
       <c r="P56" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="Q56" t="n">
-        <v>200</v>
+        <v>187.531172069825</v>
       </c>
       <c r="R56"/>
       <c r="S56"/>
@@ -17591,10 +17657,10 @@
         <v>190</v>
       </c>
       <c r="P57" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="Q57" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="R57"/>
       <c r="S57"/>
@@ -18008,7 +18074,7 @@
         <v>150</v>
       </c>
       <c r="Q59" t="n">
-        <v>500</v>
+        <v>616</v>
       </c>
       <c r="R59"/>
       <c r="S59"/>
@@ -18463,10 +18529,10 @@
         <v>183</v>
       </c>
       <c r="P61" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="Q61" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="R61"/>
       <c r="S61"/>
@@ -18895,10 +18961,10 @@
         <v>183</v>
       </c>
       <c r="P63" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q63" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="R63"/>
       <c r="S63"/>
@@ -18906,7 +18972,7 @@
         <v>40</v>
       </c>
       <c r="U63" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="V63" t="n">
         <v>120</v>
@@ -19375,10 +19441,10 @@
         <v>183</v>
       </c>
       <c r="P65" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="Q65" t="n">
-        <v>1200</v>
+        <v>1250</v>
       </c>
       <c r="R65"/>
       <c r="S65"/>
@@ -19505,7 +19571,7 @@
       <c r="CZ65"/>
       <c r="DA65"/>
       <c r="DB65" t="n">
-        <v>0.82502345</v>
+        <v>1.65</v>
       </c>
       <c r="DC65" t="n">
         <v>-1.97</v>
@@ -19899,10 +19965,10 @@
         <v>183</v>
       </c>
       <c r="P67" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q67" t="n">
-        <v>826</v>
+        <v>1000</v>
       </c>
       <c r="R67"/>
       <c r="S67"/>
@@ -19910,7 +19976,7 @@
         <v>6400</v>
       </c>
       <c r="U67" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="V67" t="n">
         <v>100</v>
@@ -20030,14 +20096,16 @@
         <v>1.513400867</v>
       </c>
       <c r="DC67" t="n">
-        <v>-7.22</v>
+        <v>-5.4</v>
       </c>
       <c r="DD67" t="n">
-        <v>-8.41</v>
-      </c>
-      <c r="DE67"/>
+        <v>-6.83</v>
+      </c>
+      <c r="DE67" t="n">
+        <v>-8.1</v>
+      </c>
       <c r="DF67" t="n">
-        <v>26.6</v>
+        <v>28.1481481481482</v>
       </c>
       <c r="DG67"/>
       <c r="DH67"/>
@@ -20175,18 +20243,22 @@
         <v>190</v>
       </c>
       <c r="P68" t="n">
-        <v>3000</v>
+        <v>750</v>
       </c>
       <c r="Q68" t="n">
-        <v>4500</v>
+        <v>2732</v>
       </c>
       <c r="R68"/>
       <c r="S68"/>
       <c r="T68" t="n">
         <v>3627.55</v>
       </c>
-      <c r="U68"/>
-      <c r="V68"/>
+      <c r="U68" t="n">
+        <v>29</v>
+      </c>
+      <c r="V68" t="n">
+        <v>80</v>
+      </c>
       <c r="W68"/>
       <c r="X68"/>
       <c r="Y68"/>
@@ -20195,9 +20267,15 @@
       <c r="AB68"/>
       <c r="AC68"/>
       <c r="AD68"/>
-      <c r="AE68"/>
-      <c r="AF68"/>
-      <c r="AG68"/>
+      <c r="AE68" t="n">
+        <v>0.184303671168695</v>
+      </c>
+      <c r="AF68" t="n">
+        <v>0.841976191188778</v>
+      </c>
+      <c r="AG68" t="n">
+        <v>0.0209122241754376</v>
+      </c>
       <c r="AH68"/>
       <c r="AI68"/>
       <c r="AJ68"/>
@@ -20206,8 +20284,12 @@
       <c r="AM68"/>
       <c r="AN68"/>
       <c r="AO68"/>
-      <c r="AP68"/>
-      <c r="AQ68"/>
+      <c r="AP68" t="n">
+        <v>0.303729951381683</v>
+      </c>
+      <c r="AQ68" t="n">
+        <v>1.02632653713226</v>
+      </c>
       <c r="AR68"/>
       <c r="AS68"/>
       <c r="AT68"/>
@@ -20290,9 +20372,7 @@
       </c>
       <c r="CZ68"/>
       <c r="DA68"/>
-      <c r="DB68" t="n">
-        <v>0.0004766</v>
-      </c>
+      <c r="DB68"/>
       <c r="DC68" t="n">
         <v>-6.81</v>
       </c>
@@ -20647,10 +20727,10 @@
         <v>190</v>
       </c>
       <c r="P70" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="Q70" t="n">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="R70"/>
       <c r="S70"/>
@@ -20889,10 +20969,10 @@
         <v>190</v>
       </c>
       <c r="P71" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="Q71" t="n">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="R71"/>
       <c r="S71"/>
@@ -21095,10 +21175,10 @@
         <v>190</v>
       </c>
       <c r="P72" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="Q72" t="n">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="R72"/>
       <c r="S72"/>
@@ -21299,10 +21379,10 @@
         <v>190</v>
       </c>
       <c r="P73" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="Q73" t="n">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="R73"/>
       <c r="S73"/>
@@ -21505,10 +21585,10 @@
         <v>190</v>
       </c>
       <c r="P74" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="Q74" t="n">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="R74"/>
       <c r="S74"/>
@@ -21709,10 +21789,10 @@
         <v>190</v>
       </c>
       <c r="P75" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="Q75" t="n">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="R75"/>
       <c r="S75"/>
@@ -22127,10 +22207,10 @@
         <v>190</v>
       </c>
       <c r="P77" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="Q77" t="n">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="R77"/>
       <c r="S77"/>
@@ -22543,10 +22623,10 @@
         <v>233</v>
       </c>
       <c r="P79" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="Q79" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="R79"/>
       <c r="S79"/>
@@ -22775,10 +22855,10 @@
         <v>183</v>
       </c>
       <c r="P80" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="Q80" t="n">
-        <v>244</v>
+        <v>350</v>
       </c>
       <c r="R80"/>
       <c r="S80"/>
@@ -23251,10 +23331,10 @@
         <v>190</v>
       </c>
       <c r="P82" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="Q82" t="n">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="R82"/>
       <c r="S82"/>
@@ -24003,7 +24083,7 @@
         <v>-1.11</v>
       </c>
       <c r="DD85" t="n">
-        <v>-3.345</v>
+        <v>-3.34</v>
       </c>
       <c r="DE85" t="n">
         <v>-5.59</v>
@@ -24739,7 +24819,7 @@
         <v>180</v>
       </c>
       <c r="J89" t="s">
-        <v>239</v>
+        <v>206</v>
       </c>
       <c r="K89" t="s">
         <v>264</v>
@@ -24757,10 +24837,10 @@
         <v>183</v>
       </c>
       <c r="P89" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="Q89" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="R89"/>
       <c r="S89"/>
@@ -24975,10 +25055,10 @@
         <v>170</v>
       </c>
       <c r="P90" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="Q90" t="n">
-        <v>639</v>
+        <v>596</v>
       </c>
       <c r="R90"/>
       <c r="S90"/>
@@ -25193,10 +25273,10 @@
         <v>190</v>
       </c>
       <c r="P91" t="n">
-        <v>40</v>
+        <v>150</v>
       </c>
       <c r="Q91" t="n">
-        <v>230</v>
+        <v>337.5</v>
       </c>
       <c r="R91"/>
       <c r="S91"/>
@@ -25255,7 +25335,7 @@
         <v>0.08</v>
       </c>
       <c r="BH91" t="n">
-        <v>2040</v>
+        <v>2044.98977505112</v>
       </c>
       <c r="BI91"/>
       <c r="BJ91" t="n">
@@ -25325,19 +25405,19 @@
       <c r="CZ91"/>
       <c r="DA91"/>
       <c r="DB91" t="n">
-        <v>0.5031513</v>
+        <v>0.73</v>
       </c>
       <c r="DC91" t="n">
-        <v>-0.926429729</v>
+        <v>-0.61151</v>
       </c>
       <c r="DD91" t="n">
-        <v>-2.947</v>
+        <v>-2.7</v>
       </c>
       <c r="DE91" t="n">
-        <v>-13.75582032</v>
+        <v>-8.33958</v>
       </c>
       <c r="DF91" t="n">
-        <v>5.92389790153517</v>
+        <v>9.83427945140249</v>
       </c>
       <c r="DG91"/>
       <c r="DH91"/>
@@ -25451,10 +25531,10 @@
         <v>170</v>
       </c>
       <c r="P92" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="Q92" t="n">
-        <v>1250</v>
+        <v>1200</v>
       </c>
       <c r="R92"/>
       <c r="S92"/>
@@ -25529,7 +25609,7 @@
         <v>0.0426310221816831</v>
       </c>
       <c r="BH92" t="n">
-        <v>2040</v>
+        <v>2044.98977505112</v>
       </c>
       <c r="BI92"/>
       <c r="BJ92" t="n">
@@ -25601,15 +25681,17 @@
       <c r="DB92" t="n">
         <v>0.73</v>
       </c>
-      <c r="DC92"/>
+      <c r="DC92" t="n">
+        <v>-1</v>
+      </c>
       <c r="DD92" t="n">
         <v>-2.7</v>
       </c>
       <c r="DE92" t="n">
-        <v>-18.56362017</v>
+        <v>-4.6</v>
       </c>
       <c r="DF92" t="n">
-        <v>7.0420149195</v>
+        <v>21.1111111111111</v>
       </c>
       <c r="DG92"/>
       <c r="DH92"/>
@@ -26864,7 +26946,7 @@
         <v>120</v>
       </c>
       <c r="Q98" t="n">
-        <v>925</v>
+        <v>938</v>
       </c>
       <c r="R98"/>
       <c r="S98"/>
@@ -27566,7 +27648,7 @@
         <v>30</v>
       </c>
       <c r="Q101" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="R101"/>
       <c r="S101"/>
@@ -27987,18 +28069,22 @@
         <v>170</v>
       </c>
       <c r="P103" t="n">
-        <v>1000</v>
+        <v>1800</v>
       </c>
       <c r="Q103" t="n">
-        <v>6500</v>
+        <v>4000</v>
       </c>
       <c r="R103"/>
       <c r="S103"/>
       <c r="T103" t="n">
         <v>27430</v>
       </c>
-      <c r="U103"/>
-      <c r="V103"/>
+      <c r="U103" t="n">
+        <v>52</v>
+      </c>
+      <c r="V103" t="n">
+        <v>154</v>
+      </c>
       <c r="W103"/>
       <c r="X103"/>
       <c r="Y103"/>
@@ -28047,7 +28133,7 @@
       <c r="BF103"/>
       <c r="BG103"/>
       <c r="BH103" t="n">
-        <v>4500.0000023278</v>
+        <v>4460.00000000001</v>
       </c>
       <c r="BI103"/>
       <c r="BJ103" t="n">
@@ -28133,17 +28219,19 @@
         <v>200</v>
       </c>
       <c r="DB103" t="n">
-        <v>1.76309933333333</v>
+        <v>1.115418936</v>
       </c>
       <c r="DC103" t="n">
-        <v>-3.9</v>
+        <v>-2.20416</v>
       </c>
       <c r="DD103" t="n">
-        <v>-4.648</v>
-      </c>
-      <c r="DE103"/>
+        <v>-4.056483</v>
+      </c>
+      <c r="DE103" t="n">
+        <v>-5.6</v>
+      </c>
       <c r="DF103" t="n">
-        <v>22.527462755583</v>
+        <v>22.3803241613268</v>
       </c>
       <c r="DG103"/>
       <c r="DH103" t="n">
@@ -28291,10 +28379,10 @@
         <v>183</v>
       </c>
       <c r="P104" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q104" t="n">
-        <v>500</v>
+        <v>508</v>
       </c>
       <c r="R104"/>
       <c r="S104"/>
@@ -28305,7 +28393,7 @@
         <v>40</v>
       </c>
       <c r="V104" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="W104"/>
       <c r="X104"/>
@@ -28764,7 +28852,7 @@
         <v>199.4</v>
       </c>
       <c r="Q106" t="n">
-        <v>4000</v>
+        <v>3390.285501</v>
       </c>
       <c r="R106" t="n">
         <v>116.4699</v>
@@ -28915,7 +29003,7 @@
         <v>38.974358974359</v>
       </c>
       <c r="DB106" t="n">
-        <v>0.84</v>
+        <v>0.8758</v>
       </c>
       <c r="DC106" t="n">
         <v>-2.5</v>
@@ -29055,10 +29143,10 @@
         <v>183</v>
       </c>
       <c r="P107" t="n">
-        <v>1600</v>
+        <v>1640</v>
       </c>
       <c r="Q107" t="n">
-        <v>3150</v>
+        <v>3199</v>
       </c>
       <c r="R107" t="n">
         <v>170.2</v>
@@ -29253,7 +29341,7 @@
         <v>38.974358974359</v>
       </c>
       <c r="DB107" t="n">
-        <v>1.62313584057143</v>
+        <v>0.8758</v>
       </c>
       <c r="DC107" t="n">
         <v>-2.5</v>
@@ -29421,10 +29509,10 @@
         <v>183</v>
       </c>
       <c r="P108" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="Q108" t="n">
-        <v>988</v>
+        <v>980</v>
       </c>
       <c r="R108"/>
       <c r="S108"/>
@@ -29435,7 +29523,7 @@
         <v>16</v>
       </c>
       <c r="V108" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="W108"/>
       <c r="X108"/>
@@ -29675,10 +29763,10 @@
         <v>183</v>
       </c>
       <c r="P109" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q109" t="n">
-        <v>700</v>
+        <v>850</v>
       </c>
       <c r="R109" t="n">
         <v>25</v>
@@ -29691,7 +29779,7 @@
         <v>40</v>
       </c>
       <c r="V109" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="W109"/>
       <c r="X109"/>
@@ -29931,10 +30019,10 @@
         <v>183</v>
       </c>
       <c r="P110" t="n">
-        <v>2000</v>
+        <v>1050</v>
       </c>
       <c r="Q110" t="n">
-        <v>4054</v>
+        <v>2600</v>
       </c>
       <c r="R110" t="n">
         <v>114.8248</v>
@@ -29943,8 +30031,12 @@
       <c r="T110" t="n">
         <v>2743.2</v>
       </c>
-      <c r="U110"/>
-      <c r="V110"/>
+      <c r="U110" t="n">
+        <v>14</v>
+      </c>
+      <c r="V110" t="n">
+        <v>119</v>
+      </c>
       <c r="W110"/>
       <c r="X110"/>
       <c r="Y110"/>
@@ -30079,17 +30171,19 @@
       <c r="CZ110"/>
       <c r="DA110"/>
       <c r="DB110" t="n">
-        <v>1.849</v>
+        <v>1.56636</v>
       </c>
       <c r="DC110" t="n">
         <v>-2.1</v>
       </c>
       <c r="DD110" t="n">
-        <v>-4.76</v>
-      </c>
-      <c r="DE110"/>
+        <v>-2.8</v>
+      </c>
+      <c r="DE110" t="n">
+        <v>-3.8</v>
+      </c>
       <c r="DF110" t="n">
-        <v>63.3</v>
+        <v>44.7058823529412</v>
       </c>
       <c r="DG110"/>
       <c r="DH110"/>
@@ -30236,7 +30330,7 @@
         <v>50</v>
       </c>
       <c r="Q111" t="n">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="R111"/>
       <c r="S111"/>
@@ -30701,10 +30795,10 @@
         <v>190</v>
       </c>
       <c r="P113" t="n">
-        <v>1625</v>
+        <v>1650</v>
       </c>
       <c r="Q113" t="n">
-        <v>2410</v>
+        <v>2416</v>
       </c>
       <c r="R113"/>
       <c r="S113"/>
@@ -31170,7 +31264,7 @@
         <v>30</v>
       </c>
       <c r="Q115" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="R115"/>
       <c r="S115"/>
@@ -31371,10 +31465,10 @@
         <v>190</v>
       </c>
       <c r="P116" t="n">
-        <v>250</v>
+        <v>550</v>
       </c>
       <c r="Q116" t="n">
-        <v>1326</v>
+        <v>1344</v>
       </c>
       <c r="R116"/>
       <c r="S116"/>
@@ -31584,7 +31678,7 @@
         <v>30</v>
       </c>
       <c r="Q117" t="n">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="R117"/>
       <c r="S117"/>
@@ -31707,7 +31801,7 @@
       <c r="CZ117"/>
       <c r="DA117"/>
       <c r="DB117" t="n">
-        <v>1.345</v>
+        <v>1.54</v>
       </c>
       <c r="DC117" t="n">
         <v>-1.06</v>
@@ -32053,7 +32147,7 @@
         <v>180</v>
       </c>
       <c r="J119" t="s">
-        <v>239</v>
+        <v>206</v>
       </c>
       <c r="K119" t="s">
         <v>264</v>
@@ -32071,10 +32165,10 @@
         <v>170</v>
       </c>
       <c r="P119" t="n">
-        <v>27.8</v>
+        <v>30</v>
       </c>
       <c r="Q119" t="n">
-        <v>589.039999999994</v>
+        <v>70</v>
       </c>
       <c r="R119"/>
       <c r="S119"/>
@@ -32501,10 +32595,10 @@
         <v>183</v>
       </c>
       <c r="P121" t="n">
-        <v>1000</v>
+        <v>560</v>
       </c>
       <c r="Q121" t="n">
-        <v>3000</v>
+        <v>1900</v>
       </c>
       <c r="R121" t="n">
         <v>49.53</v>
@@ -32513,8 +32607,12 @@
       <c r="T121" t="n">
         <v>596.9</v>
       </c>
-      <c r="U121"/>
-      <c r="V121"/>
+      <c r="U121" t="n">
+        <v>29</v>
+      </c>
+      <c r="V121" t="n">
+        <v>108</v>
+      </c>
       <c r="W121"/>
       <c r="X121"/>
       <c r="Y121"/>
@@ -32571,7 +32669,7 @@
       </c>
       <c r="BG121"/>
       <c r="BH121" t="n">
-        <v>5272.72727</v>
+        <v>11848.3412322275</v>
       </c>
       <c r="BI121"/>
       <c r="BJ121" t="n">
@@ -32647,7 +32745,7 @@
       <c r="CZ121"/>
       <c r="DA121"/>
       <c r="DB121" t="n">
-        <v>0.79</v>
+        <v>1.190638012</v>
       </c>
       <c r="DC121" t="n">
         <v>-3.66763636363636</v>
@@ -32661,7 +32759,9 @@
       <c r="DF121" t="n">
         <v>12.6015301211993</v>
       </c>
-      <c r="DG121"/>
+      <c r="DG121" t="n">
+        <v>0.256959228</v>
+      </c>
       <c r="DH121"/>
       <c r="DI121" t="n">
         <v>-1.75</v>
@@ -33017,10 +33117,10 @@
         <v>183</v>
       </c>
       <c r="P123" t="n">
-        <v>2000</v>
+        <v>1100</v>
       </c>
       <c r="Q123" t="n">
-        <v>5000</v>
+        <v>2262</v>
       </c>
       <c r="R123" t="n">
         <v>262</v>
@@ -33029,8 +33129,12 @@
       <c r="T123" t="n">
         <v>4700</v>
       </c>
-      <c r="U123"/>
-      <c r="V123"/>
+      <c r="U123" t="n">
+        <v>22</v>
+      </c>
+      <c r="V123" t="n">
+        <v>81</v>
+      </c>
       <c r="W123"/>
       <c r="X123"/>
       <c r="Y123"/>
@@ -33284,7 +33388,7 @@
         <v>910</v>
       </c>
       <c r="Q124" t="n">
-        <v>3511.00000000001</v>
+        <v>842.765109</v>
       </c>
       <c r="R124" t="n">
         <v>121</v>
@@ -33423,10 +33527,10 @@
         <v>57.1428571428571</v>
       </c>
       <c r="DB124" t="n">
-        <v>0.2182</v>
+        <v>0.28</v>
       </c>
       <c r="DC124" t="n">
-        <v>-7.21</v>
+        <v>-5.875</v>
       </c>
       <c r="DD124" t="n">
         <v>-9</v>
@@ -33435,14 +33539,16 @@
         <v>-9.37</v>
       </c>
       <c r="DF124" t="n">
-        <v>35.1851851851852</v>
-      </c>
-      <c r="DG124"/>
+        <v>21.7453505007153</v>
+      </c>
+      <c r="DG124" t="n">
+        <v>2.67</v>
+      </c>
       <c r="DH124" t="n">
         <v>-4.6</v>
       </c>
       <c r="DI124" t="n">
-        <v>-7.03</v>
+        <v>-7.2</v>
       </c>
       <c r="DJ124" t="n">
         <v>-10.2</v>
@@ -33563,10 +33669,10 @@
         <v>183</v>
       </c>
       <c r="P125" t="n">
-        <v>900</v>
+        <v>975</v>
       </c>
       <c r="Q125" t="n">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="R125"/>
       <c r="S125"/>
@@ -33769,10 +33875,10 @@
         <v>183</v>
       </c>
       <c r="P126" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q126" t="n">
-        <v>450</v>
+        <v>580</v>
       </c>
       <c r="R126"/>
       <c r="S126"/>
@@ -33793,9 +33899,15 @@
       <c r="AB126"/>
       <c r="AC126"/>
       <c r="AD126"/>
-      <c r="AE126"/>
-      <c r="AF126"/>
-      <c r="AG126"/>
+      <c r="AE126" t="n">
+        <v>0.184303671168695</v>
+      </c>
+      <c r="AF126" t="n">
+        <v>0.841976191188778</v>
+      </c>
+      <c r="AG126" t="n">
+        <v>0.0209122241754376</v>
+      </c>
       <c r="AH126"/>
       <c r="AI126"/>
       <c r="AJ126"/>
@@ -33804,8 +33916,12 @@
       <c r="AM126"/>
       <c r="AN126"/>
       <c r="AO126"/>
-      <c r="AP126"/>
-      <c r="AQ126"/>
+      <c r="AP126" t="n">
+        <v>0.303729951381683</v>
+      </c>
+      <c r="AQ126" t="n">
+        <v>1.02632653713226</v>
+      </c>
       <c r="AR126" t="n">
         <v>3.16666666666667</v>
       </c>
@@ -33833,7 +33949,7 @@
       </c>
       <c r="BG126"/>
       <c r="BH126" t="n">
-        <v>2391.667</v>
+        <v>2518.89168765743</v>
       </c>
       <c r="BI126"/>
       <c r="BJ126" t="n">
@@ -33895,13 +34011,13 @@
       <c r="CZ126"/>
       <c r="DA126"/>
       <c r="DB126" t="n">
-        <v>0.5600875</v>
+        <v>0.56</v>
       </c>
       <c r="DC126" t="n">
         <v>-4.37</v>
       </c>
       <c r="DD126" t="n">
-        <v>-6.37</v>
+        <v>-6.01444444444444</v>
       </c>
       <c r="DE126" t="n">
         <v>-7.77</v>
@@ -34041,10 +34157,10 @@
         <v>183</v>
       </c>
       <c r="P127" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q127" t="n">
-        <v>650</v>
+        <v>748</v>
       </c>
       <c r="R127"/>
       <c r="S127"/>
@@ -34297,7 +34413,7 @@
         <v>164</v>
       </c>
       <c r="J128" t="s">
-        <v>165</v>
+        <v>460</v>
       </c>
       <c r="K128" t="s">
         <v>166</v>
@@ -34315,10 +34431,10 @@
         <v>183</v>
       </c>
       <c r="P128" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q128" t="n">
-        <v>540</v>
+        <v>650</v>
       </c>
       <c r="R128"/>
       <c r="S128"/>
@@ -34326,7 +34442,7 @@
         <v>2500</v>
       </c>
       <c r="U128" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="V128" t="n">
         <v>70</v>
@@ -34339,9 +34455,15 @@
       <c r="AB128"/>
       <c r="AC128"/>
       <c r="AD128"/>
-      <c r="AE128"/>
-      <c r="AF128"/>
-      <c r="AG128"/>
+      <c r="AE128" t="n">
+        <v>0.184303671168695</v>
+      </c>
+      <c r="AF128" t="n">
+        <v>0.841976191188778</v>
+      </c>
+      <c r="AG128" t="n">
+        <v>0.0209122241754376</v>
+      </c>
       <c r="AH128"/>
       <c r="AI128"/>
       <c r="AJ128"/>
@@ -34351,10 +34473,10 @@
       <c r="AN128"/>
       <c r="AO128"/>
       <c r="AP128" t="n">
-        <v>0.928780317306519</v>
+        <v>0.303729951381683</v>
       </c>
       <c r="AQ128" t="n">
-        <v>0.555356621742249</v>
+        <v>1.02632653713226</v>
       </c>
       <c r="AR128" t="n">
         <v>2.33333333333333</v>
@@ -34569,10 +34691,10 @@
         <v>183</v>
       </c>
       <c r="P129" t="n">
-        <v>500</v>
+        <v>550</v>
       </c>
       <c r="Q129" t="n">
-        <v>1100</v>
+        <v>1140</v>
       </c>
       <c r="R129"/>
       <c r="S129"/>
@@ -35035,7 +35157,7 @@
         <v>55</v>
       </c>
       <c r="V131" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="W131"/>
       <c r="X131"/>
@@ -35091,7 +35213,7 @@
       <c r="BF131"/>
       <c r="BG131"/>
       <c r="BH131" t="n">
-        <v>2440</v>
+        <v>2439.0243902439</v>
       </c>
       <c r="BI131"/>
       <c r="BJ131" t="n">
@@ -35161,13 +35283,13 @@
       <c r="CZ131"/>
       <c r="DA131"/>
       <c r="DB131" t="n">
-        <v>0.2343383</v>
+        <v>0.28</v>
       </c>
       <c r="DC131" t="n">
         <v>-3.08</v>
       </c>
       <c r="DD131" t="n">
-        <v>-3.81</v>
+        <v>-3.6</v>
       </c>
       <c r="DE131" t="n">
         <v>-4.39</v>
@@ -35175,7 +35297,9 @@
       <c r="DF131" t="n">
         <v>58.0152671755725</v>
       </c>
-      <c r="DG131"/>
+      <c r="DG131" t="n">
+        <v>2.79</v>
+      </c>
       <c r="DH131" t="n">
         <v>-2.03</v>
       </c>
@@ -35535,18 +35659,22 @@
         <v>183</v>
       </c>
       <c r="P133" t="n">
-        <v>1200</v>
+        <v>900</v>
       </c>
       <c r="Q133" t="n">
-        <v>2000</v>
+        <v>2350</v>
       </c>
       <c r="R133"/>
       <c r="S133"/>
       <c r="T133" t="n">
         <v>2744.95709773035</v>
       </c>
-      <c r="U133"/>
-      <c r="V133"/>
+      <c r="U133" t="n">
+        <v>35</v>
+      </c>
+      <c r="V133" t="n">
+        <v>120</v>
+      </c>
       <c r="W133"/>
       <c r="X133"/>
       <c r="Y133"/>
@@ -35669,7 +35797,7 @@
         <v>43.4285714285715</v>
       </c>
       <c r="DB133" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="DC133" t="n">
         <v>-7</v>
@@ -36177,7 +36305,7 @@
       <c r="CZ135"/>
       <c r="DA135"/>
       <c r="DB135" t="n">
-        <v>0.8</v>
+        <v>0.73</v>
       </c>
       <c r="DC135" t="n">
         <v>-7.71</v>
@@ -36497,7 +36625,7 @@
         <v>180</v>
       </c>
       <c r="J137" t="s">
-        <v>460</v>
+        <v>206</v>
       </c>
       <c r="K137" t="s">
         <v>166</v>
@@ -36515,7 +36643,7 @@
         <v>183</v>
       </c>
       <c r="P137" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q137" t="n">
         <v>300</v>
@@ -36759,7 +36887,7 @@
         <v>180</v>
       </c>
       <c r="J138" t="s">
-        <v>460</v>
+        <v>165</v>
       </c>
       <c r="K138" t="s">
         <v>166</v>
@@ -36777,10 +36905,10 @@
         <v>183</v>
       </c>
       <c r="P138" t="n">
-        <v>100</v>
+        <v>350</v>
       </c>
       <c r="Q138" t="n">
-        <v>1194</v>
+        <v>1274</v>
       </c>
       <c r="R138"/>
       <c r="S138"/>
@@ -36791,7 +36919,7 @@
         <v>22</v>
       </c>
       <c r="V138" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="W138"/>
       <c r="X138"/>
@@ -37007,7 +37135,7 @@
         <v>180</v>
       </c>
       <c r="J139" t="s">
-        <v>165</v>
+        <v>206</v>
       </c>
       <c r="K139" t="s">
         <v>166</v>
@@ -37025,10 +37153,10 @@
         <v>183</v>
       </c>
       <c r="P139" t="n">
-        <v>1000</v>
+        <v>185</v>
       </c>
       <c r="Q139" t="n">
-        <v>3055.64</v>
+        <v>486</v>
       </c>
       <c r="R139"/>
       <c r="S139"/>
@@ -37473,10 +37601,10 @@
         <v>183</v>
       </c>
       <c r="P141" t="n">
-        <v>665</v>
+        <v>575</v>
       </c>
       <c r="Q141" t="n">
-        <v>2052</v>
+        <v>1362</v>
       </c>
       <c r="R141" t="n">
         <v>14.72353</v>
@@ -37489,7 +37617,7 @@
         <v>13</v>
       </c>
       <c r="V141" t="n">
-        <v>51</v>
+        <v>91</v>
       </c>
       <c r="W141"/>
       <c r="X141"/>
@@ -37603,13 +37731,13 @@
       <c r="CZ141"/>
       <c r="DA141"/>
       <c r="DB141" t="n">
-        <v>0.53</v>
+        <v>1.710288927</v>
       </c>
       <c r="DC141" t="n">
         <v>-0.907637678050247</v>
       </c>
       <c r="DD141" t="n">
-        <v>-1.59428079518203</v>
+        <v>-1.2</v>
       </c>
       <c r="DE141" t="n">
         <v>-2.02091281557024</v>
@@ -37745,10 +37873,10 @@
         <v>183</v>
       </c>
       <c r="P142" t="n">
-        <v>800</v>
+        <v>850</v>
       </c>
       <c r="Q142" t="n">
-        <v>2150</v>
+        <v>2200</v>
       </c>
       <c r="R142"/>
       <c r="S142"/>
@@ -37989,10 +38117,10 @@
         <v>183</v>
       </c>
       <c r="P143" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q143" t="n">
-        <v>350</v>
+        <v>495</v>
       </c>
       <c r="R143"/>
       <c r="S143"/>
@@ -38117,7 +38245,7 @@
       <c r="CZ143"/>
       <c r="DA143"/>
       <c r="DB143" t="n">
-        <v>0.794</v>
+        <v>0.49</v>
       </c>
       <c r="DC143" t="n">
         <v>-6.99</v>
@@ -38248,7 +38376,7 @@
         <v>200</v>
       </c>
       <c r="Q144" t="n">
-        <v>536</v>
+        <v>555</v>
       </c>
       <c r="R144"/>
       <c r="S144"/>
@@ -38365,7 +38493,7 @@
       <c r="CZ144"/>
       <c r="DA144"/>
       <c r="DB144" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="DC144" t="n">
         <v>-0.4</v>
@@ -38499,10 +38627,10 @@
         <v>183</v>
       </c>
       <c r="P145" t="n">
-        <v>1000</v>
+        <v>1150</v>
       </c>
       <c r="Q145" t="n">
-        <v>2424</v>
+        <v>2426</v>
       </c>
       <c r="R145"/>
       <c r="S145"/>
@@ -38707,10 +38835,10 @@
         <v>183</v>
       </c>
       <c r="P146" t="n">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="Q146" t="n">
-        <v>1020</v>
+        <v>1060</v>
       </c>
       <c r="R146"/>
       <c r="S146"/>
@@ -38853,13 +38981,13 @@
       <c r="CZ146"/>
       <c r="DA146"/>
       <c r="DB146" t="n">
-        <v>0.72</v>
+        <v>1.168408</v>
       </c>
       <c r="DC146" t="n">
         <v>-3.8</v>
       </c>
       <c r="DD146" t="n">
-        <v>-5.67</v>
+        <v>-5.3</v>
       </c>
       <c r="DE146" t="n">
         <v>-6.6</v>
@@ -39236,7 +39364,7 @@
         <v>60</v>
       </c>
       <c r="Q148" t="n">
-        <v>201</v>
+        <v>221</v>
       </c>
       <c r="R148"/>
       <c r="S148"/>
@@ -39256,30 +39384,14 @@
       <c r="AE148"/>
       <c r="AF148"/>
       <c r="AG148"/>
-      <c r="AH148" t="n">
-        <v>2.36476</v>
-      </c>
-      <c r="AI148" t="n">
-        <v>-0.763</v>
-      </c>
-      <c r="AJ148" t="n">
-        <v>-0.02285</v>
-      </c>
-      <c r="AK148" t="n">
-        <v>0.000074049</v>
-      </c>
-      <c r="AL148" t="n">
-        <v>-0.01018</v>
-      </c>
-      <c r="AM148" t="n">
-        <v>-0.27004</v>
-      </c>
-      <c r="AN148" t="n">
-        <v>1.09636482208082</v>
-      </c>
-      <c r="AO148" t="n">
-        <v>0.538</v>
-      </c>
+      <c r="AH148"/>
+      <c r="AI148"/>
+      <c r="AJ148"/>
+      <c r="AK148"/>
+      <c r="AL148"/>
+      <c r="AM148"/>
+      <c r="AN148"/>
+      <c r="AO148"/>
       <c r="AP148"/>
       <c r="AQ148"/>
       <c r="AR148"/>
@@ -39909,10 +40021,10 @@
         <v>183</v>
       </c>
       <c r="P151" t="n">
-        <v>1350</v>
+        <v>1400</v>
       </c>
       <c r="Q151" t="n">
-        <v>2876</v>
+        <v>2900</v>
       </c>
       <c r="R151"/>
       <c r="S151"/>
@@ -40407,10 +40519,10 @@
         <v>183</v>
       </c>
       <c r="P153" t="n">
-        <v>80</v>
+        <v>250</v>
       </c>
       <c r="Q153" t="n">
-        <v>872</v>
+        <v>1000</v>
       </c>
       <c r="R153"/>
       <c r="S153"/>
@@ -40483,7 +40595,7 @@
       </c>
       <c r="BG153"/>
       <c r="BH153" t="n">
-        <v>1700</v>
+        <v>1698.94953949973</v>
       </c>
       <c r="BI153"/>
       <c r="BJ153" t="n">
@@ -40549,7 +40661,7 @@
       <c r="CZ153"/>
       <c r="DA153"/>
       <c r="DB153" t="n">
-        <v>0.4083769</v>
+        <v>0.40837685</v>
       </c>
       <c r="DC153" t="n">
         <v>-3.06267</v>
@@ -40563,7 +40675,9 @@
       <c r="DF153" t="n">
         <v>8.3449265591562</v>
       </c>
-      <c r="DG153"/>
+      <c r="DG153" t="n">
+        <v>1.889494947</v>
+      </c>
       <c r="DH153" t="n">
         <v>-3.12248</v>
       </c>
@@ -40697,7 +40811,7 @@
         <v>170</v>
       </c>
       <c r="P154" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="Q154" t="n">
         <v>150</v>
@@ -40939,10 +41053,10 @@
         <v>183</v>
       </c>
       <c r="P155" t="n">
-        <v>80</v>
+        <v>650</v>
       </c>
       <c r="Q155" t="n">
-        <v>601</v>
+        <v>1650</v>
       </c>
       <c r="R155"/>
       <c r="S155"/>
@@ -40950,10 +41064,10 @@
         <v>2744.95709773035</v>
       </c>
       <c r="U155" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V155" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="W155"/>
       <c r="X155"/>
@@ -41167,10 +41281,10 @@
         <v>183</v>
       </c>
       <c r="P156" t="n">
-        <v>550</v>
+        <v>825</v>
       </c>
       <c r="Q156" t="n">
-        <v>1967</v>
+        <v>1988</v>
       </c>
       <c r="R156"/>
       <c r="S156"/>
@@ -41383,10 +41497,10 @@
         <v>170</v>
       </c>
       <c r="P157" t="n">
-        <v>1640</v>
+        <v>1650</v>
       </c>
       <c r="Q157" t="n">
-        <v>3026</v>
+        <v>3034</v>
       </c>
       <c r="R157" t="n">
         <v>150</v>
@@ -41410,22 +41524,44 @@
       <c r="AC157"/>
       <c r="AD157"/>
       <c r="AE157" t="n">
-        <v>0.095565</v>
+        <v>0.170586159355792</v>
       </c>
       <c r="AF157" t="n">
-        <v>1.56</v>
-      </c>
-      <c r="AG157"/>
-      <c r="AH157"/>
-      <c r="AI157"/>
-      <c r="AJ157"/>
-      <c r="AK157"/>
-      <c r="AL157"/>
-      <c r="AM157"/>
-      <c r="AN157"/>
-      <c r="AO157"/>
-      <c r="AP157"/>
-      <c r="AQ157"/>
+        <v>1.37822466400964</v>
+      </c>
+      <c r="AG157" t="n">
+        <v>0.00214453867981628</v>
+      </c>
+      <c r="AH157" t="n">
+        <v>2.36476</v>
+      </c>
+      <c r="AI157" t="n">
+        <v>-0.763</v>
+      </c>
+      <c r="AJ157" t="n">
+        <v>-0.02285</v>
+      </c>
+      <c r="AK157" t="n">
+        <v>0.000074049</v>
+      </c>
+      <c r="AL157" t="n">
+        <v>-0.01018</v>
+      </c>
+      <c r="AM157" t="n">
+        <v>-0.27004</v>
+      </c>
+      <c r="AN157" t="n">
+        <v>1.09636482208082</v>
+      </c>
+      <c r="AO157" t="n">
+        <v>0.538</v>
+      </c>
+      <c r="AP157" t="n">
+        <v>0.667239487171173</v>
+      </c>
+      <c r="AQ157" t="n">
+        <v>0.817502081394196</v>
+      </c>
       <c r="AR157" t="n">
         <v>8.52744160233958</v>
       </c>
@@ -41459,7 +41595,7 @@
       <c r="BF157"/>
       <c r="BG157"/>
       <c r="BH157" t="n">
-        <v>1975</v>
+        <v>869.565217391304</v>
       </c>
       <c r="BI157"/>
       <c r="BJ157"/>
@@ -41523,7 +41659,7 @@
       <c r="CZ157"/>
       <c r="DA157"/>
       <c r="DB157" t="n">
-        <v>0.605469915388889</v>
+        <v>0.381578947</v>
       </c>
       <c r="DC157" t="n">
         <v>-2.8</v>
@@ -41664,7 +41800,7 @@
         <v>1700</v>
       </c>
       <c r="Q158" t="n">
-        <v>5000</v>
+        <v>2680.4083689375</v>
       </c>
       <c r="R158" t="n">
         <v>121</v>
@@ -41823,7 +41959,7 @@
         <v>44.7058823529412</v>
       </c>
       <c r="DB158" t="n">
-        <v>0.18</v>
+        <v>0.22</v>
       </c>
       <c r="DC158" t="n">
         <v>-2.43</v>
@@ -41837,12 +41973,14 @@
       <c r="DF158" t="n">
         <v>32.4786324786325</v>
       </c>
-      <c r="DG158"/>
+      <c r="DG158" t="n">
+        <v>3.82</v>
+      </c>
       <c r="DH158" t="n">
         <v>-0.68</v>
       </c>
       <c r="DI158" t="n">
-        <v>-1.47</v>
+        <v>-1.65</v>
       </c>
       <c r="DJ158" t="n">
         <v>-2.5</v>
@@ -41969,7 +42107,7 @@
         <v>170</v>
       </c>
       <c r="P159" t="n">
-        <v>1400</v>
+        <v>1450</v>
       </c>
       <c r="Q159" t="n">
         <v>3100</v>
@@ -42083,7 +42221,7 @@
       <c r="CZ159"/>
       <c r="DA159"/>
       <c r="DB159" t="n">
-        <v>0.301818181818182</v>
+        <v>0.29</v>
       </c>
       <c r="DC159" t="n">
         <v>-1.68</v>
@@ -42223,10 +42361,10 @@
         <v>170</v>
       </c>
       <c r="P160" t="n">
-        <v>850</v>
+        <v>880</v>
       </c>
       <c r="Q160" t="n">
-        <v>1870</v>
+        <v>1900</v>
       </c>
       <c r="R160"/>
       <c r="S160"/>
@@ -42303,7 +42441,7 @@
         <v>0.0005</v>
       </c>
       <c r="BH160" t="n">
-        <v>1320</v>
+        <v>1982.65965862566</v>
       </c>
       <c r="BI160"/>
       <c r="BJ160" t="n">
@@ -42383,7 +42521,7 @@
       <c r="CZ160"/>
       <c r="DA160"/>
       <c r="DB160" t="n">
-        <v>0.15</v>
+        <v>0.415266667</v>
       </c>
       <c r="DC160" t="n">
         <v>-4.5</v>
@@ -42397,7 +42535,9 @@
       <c r="DF160" t="n">
         <v>43.6523207526579</v>
       </c>
-      <c r="DG160"/>
+      <c r="DG160" t="n">
+        <v>0.89</v>
+      </c>
       <c r="DH160" t="n">
         <v>-0.51103</v>
       </c>
@@ -42537,10 +42677,10 @@
         <v>170</v>
       </c>
       <c r="P161" t="n">
-        <v>970</v>
+        <v>1000</v>
       </c>
       <c r="Q161" t="n">
-        <v>2210</v>
+        <v>2250</v>
       </c>
       <c r="R161"/>
       <c r="S161"/>
@@ -42627,7 +42767,7 @@
       </c>
       <c r="BG161"/>
       <c r="BH161" t="n">
-        <v>1270</v>
+        <v>3052.50305250305</v>
       </c>
       <c r="BI161"/>
       <c r="BJ161" t="n">
@@ -42707,7 +42847,7 @@
       <c r="CZ161"/>
       <c r="DA161"/>
       <c r="DB161" t="n">
-        <v>0.00028111988</v>
+        <v>0.3658</v>
       </c>
       <c r="DC161" t="n">
         <v>-1.75</v>
@@ -42849,7 +42989,7 @@
         <v>170</v>
       </c>
       <c r="P162" t="n">
-        <v>1150</v>
+        <v>1200</v>
       </c>
       <c r="Q162" t="n">
         <v>2600</v>
@@ -42927,7 +43067,7 @@
       <c r="BF162"/>
       <c r="BG162"/>
       <c r="BH162" t="n">
-        <v>1010</v>
+        <v>1013.17122593718</v>
       </c>
       <c r="BI162"/>
       <c r="BJ162" t="n">
@@ -42997,7 +43137,7 @@
       <c r="CZ162"/>
       <c r="DA162"/>
       <c r="DB162" t="n">
-        <v>0.794</v>
+        <v>1</v>
       </c>
       <c r="DC162" t="n">
         <v>-3.01</v>
@@ -43149,10 +43289,10 @@
         <v>183</v>
       </c>
       <c r="P163" t="n">
-        <v>900</v>
+        <v>920</v>
       </c>
       <c r="Q163" t="n">
-        <v>1850</v>
+        <v>1869</v>
       </c>
       <c r="R163" t="n">
         <v>200</v>
@@ -43223,7 +43363,7 @@
       <c r="BF163"/>
       <c r="BG163"/>
       <c r="BH163" t="n">
-        <v>1620</v>
+        <v>1615.50888529887</v>
       </c>
       <c r="BI163"/>
       <c r="BJ163" t="n">
@@ -43319,7 +43459,9 @@
       <c r="DF163" t="n">
         <v>28.8177881589225</v>
       </c>
-      <c r="DG163"/>
+      <c r="DG163" t="n">
+        <v>1.7</v>
+      </c>
       <c r="DH163" t="n">
         <v>-0.47</v>
       </c>
@@ -43479,35 +43621,33 @@
       <c r="AB164"/>
       <c r="AC164"/>
       <c r="AD164"/>
-      <c r="AE164"/>
-      <c r="AF164"/>
-      <c r="AG164"/>
-      <c r="AH164" t="n">
-        <v>2.36476</v>
-      </c>
-      <c r="AI164" t="n">
-        <v>-0.763</v>
-      </c>
-      <c r="AJ164" t="n">
-        <v>-0.02285</v>
-      </c>
-      <c r="AK164" t="n">
-        <v>0.000074049</v>
-      </c>
-      <c r="AL164" t="n">
-        <v>-0.01018</v>
-      </c>
-      <c r="AM164" t="n">
-        <v>-0.27004</v>
-      </c>
+      <c r="AE164" t="n">
+        <v>1.76400781306929</v>
+      </c>
+      <c r="AF164" t="n">
+        <v>0.582063431740351</v>
+      </c>
+      <c r="AG164" t="n">
+        <v>-0.0287078067206654</v>
+      </c>
+      <c r="AH164"/>
+      <c r="AI164"/>
+      <c r="AJ164"/>
+      <c r="AK164"/>
+      <c r="AL164"/>
+      <c r="AM164"/>
       <c r="AN164" t="n">
-        <v>1.09636482208082</v>
+        <v>0.841894979460939</v>
       </c>
       <c r="AO164" t="n">
-        <v>0.538</v>
-      </c>
-      <c r="AP164"/>
-      <c r="AQ164"/>
+        <v>0.6353</v>
+      </c>
+      <c r="AP164" t="n">
+        <v>0.402596145868301</v>
+      </c>
+      <c r="AQ164" t="n">
+        <v>1.16842377185822</v>
+      </c>
       <c r="AR164"/>
       <c r="AS164"/>
       <c r="AT164"/>
@@ -43835,7 +43975,7 @@
       </c>
       <c r="BG165"/>
       <c r="BH165" t="n">
-        <v>1800</v>
+        <v>2128.01726247603</v>
       </c>
       <c r="BI165"/>
       <c r="BJ165" t="n">
@@ -43923,7 +44063,7 @@
       <c r="CZ165"/>
       <c r="DA165"/>
       <c r="DB165" t="n">
-        <v>1.48471741467857</v>
+        <v>0.439943228</v>
       </c>
       <c r="DC165" t="n">
         <v>-2.62</v>
@@ -43937,12 +44077,14 @@
       <c r="DF165" t="n">
         <v>35.6302331904999</v>
       </c>
-      <c r="DG165"/>
+      <c r="DG165" t="n">
+        <v>0.203468369</v>
+      </c>
       <c r="DH165" t="n">
         <v>-1.01</v>
       </c>
       <c r="DI165" t="n">
-        <v>-1.65</v>
+        <v>-1.951988</v>
       </c>
       <c r="DJ165" t="n">
         <v>-2.916418083</v>
@@ -44081,10 +44223,10 @@
         <v>170</v>
       </c>
       <c r="P166" t="n">
-        <v>1030</v>
+        <v>1050</v>
       </c>
       <c r="Q166" t="n">
-        <v>2060</v>
+        <v>2100</v>
       </c>
       <c r="R166" t="n">
         <v>100</v>
@@ -44359,10 +44501,10 @@
         <v>183</v>
       </c>
       <c r="P167" t="n">
-        <v>100</v>
+        <v>825</v>
       </c>
       <c r="Q167" t="n">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="R167"/>
       <c r="S167"/>
@@ -44661,7 +44803,7 @@
         <v>0.09483</v>
       </c>
       <c r="BH168" t="n">
-        <v>3560</v>
+        <v>3558.71886120996</v>
       </c>
       <c r="BI168"/>
       <c r="BJ168"/>
@@ -44731,7 +44873,7 @@
       <c r="CZ168"/>
       <c r="DA168"/>
       <c r="DB168" t="n">
-        <v>0.718</v>
+        <v>0.73</v>
       </c>
       <c r="DC168" t="n">
         <v>-5.62</v>
@@ -44865,10 +45007,10 @@
         <v>183</v>
       </c>
       <c r="P169" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q169" t="n">
-        <v>647</v>
+        <v>721</v>
       </c>
       <c r="R169"/>
       <c r="S169"/>
@@ -45121,10 +45263,10 @@
         <v>170</v>
       </c>
       <c r="P170" t="n">
-        <v>3000</v>
+        <v>2150</v>
       </c>
       <c r="Q170" t="n">
-        <v>5054</v>
+        <v>3400</v>
       </c>
       <c r="R170" t="n">
         <v>400</v>
@@ -45133,8 +45275,12 @@
       <c r="T170" t="n">
         <v>2743.2</v>
       </c>
-      <c r="U170"/>
-      <c r="V170"/>
+      <c r="U170" t="n">
+        <v>41</v>
+      </c>
+      <c r="V170" t="n">
+        <v>124</v>
+      </c>
       <c r="W170"/>
       <c r="X170"/>
       <c r="Y170"/>
@@ -45596,15 +45742,19 @@
         <v>2000</v>
       </c>
       <c r="Q172" t="n">
-        <v>5791.2</v>
+        <v>3550</v>
       </c>
       <c r="R172"/>
       <c r="S172"/>
       <c r="T172" t="n">
         <v>12030</v>
       </c>
-      <c r="U172"/>
-      <c r="V172"/>
+      <c r="U172" t="n">
+        <v>36</v>
+      </c>
+      <c r="V172" t="n">
+        <v>116</v>
+      </c>
       <c r="W172"/>
       <c r="X172"/>
       <c r="Y172"/>
@@ -45657,7 +45807,7 @@
       <c r="BF172"/>
       <c r="BG172"/>
       <c r="BH172" t="n">
-        <v>4510</v>
+        <v>3597.12230215827</v>
       </c>
       <c r="BI172"/>
       <c r="BJ172" t="n">
@@ -45741,13 +45891,13 @@
         <v>98.7012987012987</v>
       </c>
       <c r="DB172" t="n">
-        <v>1.787140872</v>
+        <v>1.114299739</v>
       </c>
       <c r="DC172" t="n">
         <v>-1.77</v>
       </c>
       <c r="DD172" t="n">
-        <v>-2.13</v>
+        <v>-1.81</v>
       </c>
       <c r="DE172" t="n">
         <v>-2.2</v>
@@ -45755,7 +45905,9 @@
       <c r="DF172" t="n">
         <v>176.744186046512</v>
       </c>
-      <c r="DG172"/>
+      <c r="DG172" t="n">
+        <v>0.737</v>
+      </c>
       <c r="DH172" t="n">
         <v>-0.2</v>
       </c>
@@ -45885,7 +46037,7 @@
         <v>180</v>
       </c>
       <c r="J173" t="s">
-        <v>165</v>
+        <v>460</v>
       </c>
       <c r="K173" t="s">
         <v>166</v>
@@ -45906,7 +46058,7 @@
         <v>100</v>
       </c>
       <c r="Q173" t="n">
-        <v>2000</v>
+        <v>2100</v>
       </c>
       <c r="R173" t="n">
         <v>32.9192307692308</v>
@@ -45916,10 +46068,10 @@
         <v>9354.99999999998</v>
       </c>
       <c r="U173" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="V173" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="W173"/>
       <c r="X173"/>
@@ -45969,7 +46121,7 @@
       <c r="BF173"/>
       <c r="BG173"/>
       <c r="BH173" t="n">
-        <v>7530.328</v>
+        <v>5291.00529100529</v>
       </c>
       <c r="BI173"/>
       <c r="BJ173" t="n">
@@ -46042,28 +46194,32 @@
         <v>-2.85</v>
       </c>
       <c r="CY173" t="n">
-        <v>-5.53</v>
-      </c>
-      <c r="CZ173"/>
+        <v>-3.99</v>
+      </c>
+      <c r="CZ173" t="n">
+        <v>-4.99</v>
+      </c>
       <c r="DA173" t="n">
         <v>35.5140186915888</v>
       </c>
       <c r="DB173" t="n">
-        <v>2.24</v>
+        <v>1.275745765</v>
       </c>
       <c r="DC173" t="n">
-        <v>-4.4</v>
+        <v>-4.39</v>
       </c>
       <c r="DD173" t="n">
-        <v>-5.55</v>
+        <v>-5.36</v>
       </c>
       <c r="DE173" t="n">
         <v>-6.53398</v>
       </c>
       <c r="DF173" t="n">
-        <v>35.6142044442778</v>
-      </c>
-      <c r="DG173"/>
+        <v>35.4480918665286</v>
+      </c>
+      <c r="DG173" t="n">
+        <v>0.82</v>
+      </c>
       <c r="DH173" t="n">
         <v>-0.79</v>
       </c>
@@ -46217,7 +46373,7 @@
         <v>183</v>
       </c>
       <c r="P174" t="n">
-        <v>1640</v>
+        <v>1650</v>
       </c>
       <c r="Q174" t="n">
         <v>3300</v>
@@ -46244,25 +46400,43 @@
       <c r="AC174"/>
       <c r="AD174"/>
       <c r="AE174" t="n">
-        <v>0.3021</v>
+        <v>0.170586159355792</v>
       </c>
       <c r="AF174" t="n">
-        <v>1.308</v>
-      </c>
-      <c r="AG174"/>
-      <c r="AH174"/>
-      <c r="AI174"/>
-      <c r="AJ174"/>
-      <c r="AK174"/>
-      <c r="AL174"/>
-      <c r="AM174"/>
-      <c r="AN174"/>
-      <c r="AO174"/>
+        <v>1.37822466400964</v>
+      </c>
+      <c r="AG174" t="n">
+        <v>0.00214453867981628</v>
+      </c>
+      <c r="AH174" t="n">
+        <v>2.36476</v>
+      </c>
+      <c r="AI174" t="n">
+        <v>-0.763</v>
+      </c>
+      <c r="AJ174" t="n">
+        <v>-0.02285</v>
+      </c>
+      <c r="AK174" t="n">
+        <v>0.000074049</v>
+      </c>
+      <c r="AL174" t="n">
+        <v>-0.01018</v>
+      </c>
+      <c r="AM174" t="n">
+        <v>-0.27004</v>
+      </c>
+      <c r="AN174" t="n">
+        <v>1.09636482208082</v>
+      </c>
+      <c r="AO174" t="n">
+        <v>0.538</v>
+      </c>
       <c r="AP174" t="n">
-        <v>0.448119103908539</v>
+        <v>0.667239487171173</v>
       </c>
       <c r="AQ174" t="n">
-        <v>0.906015455722809</v>
+        <v>0.817502081394196</v>
       </c>
       <c r="AR174" t="n">
         <v>5.38045190862213</v>
@@ -46291,7 +46465,7 @@
       <c r="BF174"/>
       <c r="BG174"/>
       <c r="BH174" t="n">
-        <v>4500</v>
+        <v>7389.9998522</v>
       </c>
       <c r="BI174"/>
       <c r="BJ174" t="n">
@@ -46369,7 +46543,7 @@
       <c r="CZ174"/>
       <c r="DA174"/>
       <c r="DB174" t="n">
-        <v>0.855972214285714</v>
+        <v>0.345397</v>
       </c>
       <c r="DC174" t="n">
         <v>-2.7</v>
@@ -46381,7 +46555,9 @@
       <c r="DF174" t="n">
         <v>34</v>
       </c>
-      <c r="DG174"/>
+      <c r="DG174" t="n">
+        <v>3.3</v>
+      </c>
       <c r="DH174" t="n">
         <v>-1.56</v>
       </c>
@@ -46525,10 +46701,10 @@
         <v>183</v>
       </c>
       <c r="P175" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q175" t="n">
-        <v>1276</v>
+        <v>1457</v>
       </c>
       <c r="R175"/>
       <c r="S175"/>
@@ -46794,7 +46970,7 @@
         <v>66</v>
       </c>
       <c r="Q176" t="n">
-        <v>3050</v>
+        <v>1997.43700339412</v>
       </c>
       <c r="R176" t="n">
         <v>152</v>
@@ -46983,23 +47159,25 @@
         <v>42.9378531073446</v>
       </c>
       <c r="DB176" t="n">
-        <v>0.758037552</v>
+        <v>0.657757582</v>
       </c>
       <c r="DC176" t="n">
         <v>-3.61</v>
       </c>
       <c r="DD176" t="n">
-        <v>-4.74</v>
+        <v>-4.54</v>
       </c>
       <c r="DE176" t="n">
-        <v>-6.84891772633333</v>
+        <v>-4.97</v>
       </c>
       <c r="DF176" t="n">
-        <v>23.4646281324463</v>
-      </c>
-      <c r="DG176"/>
+        <v>55.8823529411765</v>
+      </c>
+      <c r="DG176" t="n">
+        <v>4.82</v>
+      </c>
       <c r="DH176" t="n">
-        <v>-1.19</v>
+        <v>-0.2</v>
       </c>
       <c r="DI176" t="n">
         <v>-1.23</v>
@@ -47008,7 +47186,7 @@
         <v>-2.3</v>
       </c>
       <c r="DK176" t="n">
-        <v>68.4684684684685</v>
+        <v>36.1904761904762</v>
       </c>
       <c r="DL176" t="n">
         <v>60.1145911283347</v>
@@ -47125,7 +47303,7 @@
         <v>183</v>
       </c>
       <c r="P177" t="n">
-        <v>1200</v>
+        <v>1270</v>
       </c>
       <c r="Q177" t="n">
         <v>2150</v>
@@ -47536,16 +47714,16 @@
         <v>0.29</v>
       </c>
       <c r="DC178" t="n">
-        <v>-4.048237444</v>
+        <v>-3.84683</v>
       </c>
       <c r="DD178" t="n">
         <v>-7</v>
       </c>
       <c r="DE178" t="n">
-        <v>-11.8239720366667</v>
+        <v>-10.0732</v>
       </c>
       <c r="DF178" t="n">
-        <v>9.77399615358215</v>
+        <v>12.2061490081701</v>
       </c>
       <c r="DG178"/>
       <c r="DH178"/>
@@ -47663,10 +47841,10 @@
         <v>183</v>
       </c>
       <c r="P179" t="n">
-        <v>530</v>
+        <v>700</v>
       </c>
       <c r="Q179" t="n">
-        <v>1680</v>
+        <v>1750</v>
       </c>
       <c r="R179"/>
       <c r="S179"/>
@@ -48171,10 +48349,10 @@
         <v>183</v>
       </c>
       <c r="P181" t="n">
-        <v>48</v>
+        <v>550</v>
       </c>
       <c r="Q181" t="n">
-        <v>415</v>
+        <v>1280</v>
       </c>
       <c r="R181" t="n">
         <v>200</v>
@@ -48183,8 +48361,12 @@
       <c r="T181" t="n">
         <v>7000</v>
       </c>
-      <c r="U181"/>
-      <c r="V181"/>
+      <c r="U181" t="n">
+        <v>15</v>
+      </c>
+      <c r="V181" t="n">
+        <v>70</v>
+      </c>
       <c r="W181" t="n">
         <v>1.85748624915521</v>
       </c>
@@ -48257,7 +48439,7 @@
         <v>0.00026</v>
       </c>
       <c r="BH181" t="n">
-        <v>1002.51204726923</v>
+        <v>1108.26238532802</v>
       </c>
       <c r="BI181"/>
       <c r="BJ181" t="n">
@@ -48353,7 +48535,7 @@
       <c r="CZ181"/>
       <c r="DA181"/>
       <c r="DB181" t="n">
-        <v>11.4</v>
+        <v>0.8268</v>
       </c>
       <c r="DC181" t="n">
         <v>-4.3</v>
@@ -48367,12 +48549,14 @@
       <c r="DF181" t="n">
         <v>21.1111111111111</v>
       </c>
-      <c r="DG181"/>
+      <c r="DG181" t="n">
+        <v>0.47</v>
+      </c>
       <c r="DH181" t="n">
         <v>-0.43456</v>
       </c>
       <c r="DI181" t="n">
-        <v>-5</v>
+        <v>-2.39</v>
       </c>
       <c r="DJ181" t="n">
         <v>-7.03</v>
@@ -48741,7 +48925,7 @@
         <v>183</v>
       </c>
       <c r="P183" t="n">
-        <v>1150</v>
+        <v>1210</v>
       </c>
       <c r="Q183" t="n">
         <v>2600</v>
@@ -48905,7 +49089,7 @@
       <c r="CZ183"/>
       <c r="DA183"/>
       <c r="DB183" t="n">
-        <v>0.644812885</v>
+        <v>0.63002894</v>
       </c>
       <c r="DC183" t="n">
         <v>-2.5</v>
@@ -49061,10 +49245,10 @@
         <v>183</v>
       </c>
       <c r="P184" t="n">
-        <v>2000</v>
+        <v>820</v>
       </c>
       <c r="Q184" t="n">
-        <v>2500</v>
+        <v>2100</v>
       </c>
       <c r="R184" t="n">
         <v>200</v>
@@ -49073,8 +49257,12 @@
       <c r="T184" t="n">
         <v>1612.5</v>
       </c>
-      <c r="U184"/>
-      <c r="V184"/>
+      <c r="U184" t="n">
+        <v>30</v>
+      </c>
+      <c r="V184" t="n">
+        <v>90</v>
+      </c>
       <c r="W184"/>
       <c r="X184"/>
       <c r="Y184"/>
@@ -49215,19 +49403,17 @@
       <c r="CZ184"/>
       <c r="DA184"/>
       <c r="DB184" t="n">
-        <v>0.93</v>
+        <v>1.040407684</v>
       </c>
       <c r="DC184" t="n">
         <v>-4.08</v>
       </c>
       <c r="DD184" t="n">
-        <v>-5.1</v>
-      </c>
-      <c r="DE184" t="n">
-        <v>-6.84891772633333</v>
-      </c>
+        <v>-4.81</v>
+      </c>
+      <c r="DE184"/>
       <c r="DF184" t="n">
-        <v>27.4475472048933</v>
+        <v>82.4</v>
       </c>
       <c r="DG184"/>
       <c r="DH184"/>
@@ -49363,10 +49549,10 @@
         <v>183</v>
       </c>
       <c r="P185" t="n">
-        <v>850</v>
+        <v>940</v>
       </c>
       <c r="Q185" t="n">
-        <v>2050</v>
+        <v>2090</v>
       </c>
       <c r="R185"/>
       <c r="S185"/>
@@ -49639,10 +49825,10 @@
         <v>183</v>
       </c>
       <c r="P186" t="n">
-        <v>1100</v>
+        <v>1290</v>
       </c>
       <c r="Q186" t="n">
-        <v>2600</v>
+        <v>2620</v>
       </c>
       <c r="R186"/>
       <c r="S186"/>
@@ -49791,7 +49977,7 @@
         <v>-4.3</v>
       </c>
       <c r="DD186" t="n">
-        <v>-6.88</v>
+        <v>-4.74</v>
       </c>
       <c r="DE186"/>
       <c r="DF186" t="n">
@@ -49939,7 +50125,7 @@
         <v>190</v>
       </c>
       <c r="P187" t="n">
-        <v>1900</v>
+        <v>2000</v>
       </c>
       <c r="Q187" t="n">
         <v>3861</v>
@@ -50009,7 +50195,7 @@
       <c r="BF187"/>
       <c r="BG187"/>
       <c r="BH187" t="n">
-        <v>5730</v>
+        <v>5725.24546989952</v>
       </c>
       <c r="BI187"/>
       <c r="BJ187" t="n">
@@ -50085,7 +50271,7 @@
       <c r="CZ187"/>
       <c r="DA187"/>
       <c r="DB187" t="n">
-        <v>27.35</v>
+        <v>0.8</v>
       </c>
       <c r="DC187" t="n">
         <v>-2.14</v>
@@ -50099,7 +50285,9 @@
       <c r="DF187" t="n">
         <v>30.6451612903226</v>
       </c>
-      <c r="DG187"/>
+      <c r="DG187" t="n">
+        <v>2.42</v>
+      </c>
       <c r="DH187" t="n">
         <v>-0.1</v>
       </c>
@@ -50251,10 +50439,10 @@
         <v>183</v>
       </c>
       <c r="P188" t="n">
-        <v>750</v>
+        <v>780</v>
       </c>
       <c r="Q188" t="n">
-        <v>1550</v>
+        <v>1570</v>
       </c>
       <c r="R188"/>
       <c r="S188"/>
@@ -50419,7 +50607,7 @@
       <c r="CZ188"/>
       <c r="DA188"/>
       <c r="DB188" t="n">
-        <v>13.62</v>
+        <v>1.03</v>
       </c>
       <c r="DC188" t="n">
         <v>-3.7</v>
@@ -50779,7 +50967,7 @@
         <v>180</v>
       </c>
       <c r="J190" t="s">
-        <v>206</v>
+        <v>460</v>
       </c>
       <c r="K190" t="s">
         <v>166</v>
@@ -50797,18 +50985,22 @@
         <v>183</v>
       </c>
       <c r="P190" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q190" t="n">
-        <v>250</v>
+        <v>645</v>
       </c>
       <c r="R190"/>
       <c r="S190"/>
       <c r="T190" t="n">
         <v>386.08</v>
       </c>
-      <c r="U190"/>
-      <c r="V190"/>
+      <c r="U190" t="n">
+        <v>38</v>
+      </c>
+      <c r="V190" t="n">
+        <v>100</v>
+      </c>
       <c r="W190"/>
       <c r="X190"/>
       <c r="Y190"/>
@@ -50929,10 +51121,10 @@
       <c r="CZ190"/>
       <c r="DA190"/>
       <c r="DB190" t="n">
-        <v>1.45</v>
+        <v>1.063</v>
       </c>
       <c r="DC190" t="n">
-        <v>-7.49</v>
+        <v>-7.41</v>
       </c>
       <c r="DD190" t="n">
         <v>-8.09</v>
@@ -50941,14 +51133,16 @@
         <v>-9.82749</v>
       </c>
       <c r="DF190" t="n">
-        <v>32.513508079179</v>
-      </c>
-      <c r="DG190"/>
+        <v>31.4375654087504</v>
+      </c>
+      <c r="DG190" t="n">
+        <v>2.82</v>
+      </c>
       <c r="DH190" t="n">
         <v>-0.57629</v>
       </c>
       <c r="DI190" t="n">
-        <v>-2.34</v>
+        <v>-2.33859</v>
       </c>
       <c r="DJ190" t="n">
         <v>-6.52125</v>
@@ -51141,7 +51335,7 @@
       </c>
       <c r="BG191"/>
       <c r="BH191" t="n">
-        <v>5200</v>
+        <v>1300.39011703511</v>
       </c>
       <c r="BI191"/>
       <c r="BJ191" t="n">
@@ -51204,18 +51398,18 @@
       </c>
       <c r="CX191"/>
       <c r="CY191" t="n">
-        <v>-2.05</v>
+        <v>-1.95</v>
       </c>
       <c r="CZ191"/>
       <c r="DA191"/>
       <c r="DB191" t="n">
-        <v>0.21</v>
+        <v>0.364</v>
       </c>
       <c r="DC191" t="n">
         <v>-0.92</v>
       </c>
       <c r="DD191" t="n">
-        <v>-2.93</v>
+        <v>-3.01</v>
       </c>
       <c r="DE191" t="n">
         <v>-5</v>
@@ -51223,7 +51417,9 @@
       <c r="DF191" t="n">
         <v>18.6274509803922</v>
       </c>
-      <c r="DG191"/>
+      <c r="DG191" t="n">
+        <v>2.41</v>
+      </c>
       <c r="DH191" t="n">
         <v>-1.11</v>
       </c>
@@ -51345,10 +51541,10 @@
         <v>183</v>
       </c>
       <c r="P192" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q192" t="n">
-        <v>1000</v>
+        <v>1124</v>
       </c>
       <c r="R192"/>
       <c r="S192"/>
@@ -51572,7 +51768,7 @@
         <v>50</v>
       </c>
       <c r="Q193" t="n">
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="R193"/>
       <c r="S193"/>
@@ -51801,7 +51997,7 @@
         <v>180</v>
       </c>
       <c r="J194" t="s">
-        <v>206</v>
+        <v>165</v>
       </c>
       <c r="K194" t="s">
         <v>166</v>
@@ -51819,18 +52015,22 @@
         <v>190</v>
       </c>
       <c r="P194" t="n">
-        <v>196.081081081081</v>
+        <v>1450</v>
       </c>
       <c r="Q194" t="n">
-        <v>422.378378378378</v>
+        <v>2897</v>
       </c>
       <c r="R194"/>
       <c r="S194"/>
       <c r="T194" t="n">
         <v>2247.3</v>
       </c>
-      <c r="U194"/>
-      <c r="V194"/>
+      <c r="U194" t="n">
+        <v>41</v>
+      </c>
+      <c r="V194" t="n">
+        <v>130</v>
+      </c>
       <c r="W194"/>
       <c r="X194"/>
       <c r="Y194"/>
@@ -52169,7 +52369,7 @@
       <c r="CZ195"/>
       <c r="DA195"/>
       <c r="DB195" t="n">
-        <v>10.61</v>
+        <v>3.315734</v>
       </c>
       <c r="DC195"/>
       <c r="DD195" t="n">
@@ -52753,7 +52953,7 @@
         <v>180</v>
       </c>
       <c r="J198" t="s">
-        <v>239</v>
+        <v>206</v>
       </c>
       <c r="K198" t="s">
         <v>207</v>
@@ -52771,10 +52971,10 @@
         <v>183</v>
       </c>
       <c r="P198" t="n">
-        <v>84</v>
+        <v>40</v>
       </c>
       <c r="Q198" t="n">
-        <v>144.62</v>
+        <v>120</v>
       </c>
       <c r="R198"/>
       <c r="S198"/>
@@ -52993,10 +53193,10 @@
         <v>190</v>
       </c>
       <c r="P199" t="n">
-        <v>630</v>
+        <v>800</v>
       </c>
       <c r="Q199" t="n">
-        <v>2156</v>
+        <v>2200</v>
       </c>
       <c r="R199"/>
       <c r="S199"/>
@@ -53004,7 +53204,7 @@
         <v>2747.28</v>
       </c>
       <c r="U199" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="V199" t="n">
         <v>110</v>
@@ -53057,7 +53257,7 @@
       <c r="BF199"/>
       <c r="BG199"/>
       <c r="BH199" t="n">
-        <v>4219.5755</v>
+        <v>2873.5632183908</v>
       </c>
       <c r="BI199"/>
       <c r="BJ199" t="n">
@@ -53131,13 +53331,13 @@
       <c r="CZ199"/>
       <c r="DA199"/>
       <c r="DB199" t="n">
-        <v>2.5</v>
+        <v>2.44</v>
       </c>
       <c r="DC199" t="n">
-        <v>-1.72</v>
+        <v>-1.64</v>
       </c>
       <c r="DD199" t="n">
-        <v>-1.99</v>
+        <v>-1.97</v>
       </c>
       <c r="DE199"/>
       <c r="DF199" t="n">
@@ -53515,10 +53715,10 @@
         <v>190</v>
       </c>
       <c r="P201" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="Q201" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="R201"/>
       <c r="S201"/>
@@ -53657,7 +53857,7 @@
       <c r="CZ201"/>
       <c r="DA201"/>
       <c r="DB201" t="n">
-        <v>0.313457120777778</v>
+        <v>0.68</v>
       </c>
       <c r="DC201" t="n">
         <v>-7.48</v>
@@ -53666,10 +53866,10 @@
         <v>-9.4</v>
       </c>
       <c r="DE201" t="n">
-        <v>-15.0056887222222</v>
+        <v>-12</v>
       </c>
       <c r="DF201" t="n">
-        <v>10.098743491155</v>
+        <v>16.8141592920354</v>
       </c>
       <c r="DG201"/>
       <c r="DH201"/>
@@ -53761,7 +53961,7 @@
         <v>180</v>
       </c>
       <c r="J202" t="s">
-        <v>206</v>
+        <v>460</v>
       </c>
       <c r="K202" t="s">
         <v>166</v>
@@ -53779,18 +53979,22 @@
         <v>183</v>
       </c>
       <c r="P202" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="Q202" t="n">
-        <v>1100</v>
+        <v>1050</v>
       </c>
       <c r="R202"/>
       <c r="S202"/>
       <c r="T202" t="n">
         <v>589.28</v>
       </c>
-      <c r="U202"/>
-      <c r="V202"/>
+      <c r="U202" t="n">
+        <v>29</v>
+      </c>
+      <c r="V202" t="n">
+        <v>90</v>
+      </c>
       <c r="W202"/>
       <c r="X202"/>
       <c r="Y202"/>
@@ -53802,30 +54006,14 @@
       <c r="AE202"/>
       <c r="AF202"/>
       <c r="AG202"/>
-      <c r="AH202" t="n">
-        <v>2.36476</v>
-      </c>
-      <c r="AI202" t="n">
-        <v>-0.763</v>
-      </c>
-      <c r="AJ202" t="n">
-        <v>-0.02285</v>
-      </c>
-      <c r="AK202" t="n">
-        <v>0.000074049</v>
-      </c>
-      <c r="AL202" t="n">
-        <v>-0.01018</v>
-      </c>
-      <c r="AM202" t="n">
-        <v>-0.27004</v>
-      </c>
-      <c r="AN202" t="n">
-        <v>1.09636482208082</v>
-      </c>
-      <c r="AO202" t="n">
-        <v>0.538</v>
-      </c>
+      <c r="AH202"/>
+      <c r="AI202"/>
+      <c r="AJ202"/>
+      <c r="AK202"/>
+      <c r="AL202"/>
+      <c r="AM202"/>
+      <c r="AN202"/>
+      <c r="AO202"/>
       <c r="AP202"/>
       <c r="AQ202"/>
       <c r="AR202" t="n">
@@ -53917,7 +54105,7 @@
       <c r="CZ202"/>
       <c r="DA202"/>
       <c r="DB202" t="n">
-        <v>10.53</v>
+        <v>2.639193</v>
       </c>
       <c r="DC202" t="n">
         <v>-1.36</v>
@@ -53931,7 +54119,9 @@
       <c r="DF202" t="n">
         <v>101.333333333333</v>
       </c>
-      <c r="DG202"/>
+      <c r="DG202" t="n">
+        <v>25.44</v>
+      </c>
       <c r="DH202"/>
       <c r="DI202" t="n">
         <v>-0.53</v>
@@ -54065,10 +54255,10 @@
         <v>183</v>
       </c>
       <c r="P203" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="Q203" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="R203"/>
       <c r="S203"/>
@@ -54285,10 +54475,10 @@
         <v>190</v>
       </c>
       <c r="P204" t="n">
-        <v>687.5</v>
+        <v>130</v>
       </c>
       <c r="Q204" t="n">
-        <v>2104.3</v>
+        <v>130</v>
       </c>
       <c r="R204"/>
       <c r="S204"/>
@@ -55129,10 +55319,10 @@
         <v>190</v>
       </c>
       <c r="P208" t="n">
-        <v>690</v>
+        <v>1300</v>
       </c>
       <c r="Q208" t="n">
-        <v>1288</v>
+        <v>1300</v>
       </c>
       <c r="R208"/>
       <c r="S208"/>
@@ -55335,10 +55525,10 @@
         <v>183</v>
       </c>
       <c r="P209" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="Q209" t="n">
-        <v>1545</v>
+        <v>1595</v>
       </c>
       <c r="R209" t="n">
         <v>30.63799</v>
@@ -55348,10 +55538,10 @@
         <v>873.76</v>
       </c>
       <c r="U209" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="V209" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="W209"/>
       <c r="X209"/>
@@ -55463,7 +55653,7 @@
       <c r="CZ209"/>
       <c r="DA209"/>
       <c r="DB209" t="n">
-        <v>0.11803715</v>
+        <v>0.1038128</v>
       </c>
       <c r="DC209" t="n">
         <v>-2.65</v>
@@ -55617,10 +55807,10 @@
         <v>190</v>
       </c>
       <c r="P210" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="Q210" t="n">
-        <v>269</v>
+        <v>300</v>
       </c>
       <c r="R210"/>
       <c r="S210"/>
@@ -56095,10 +56285,10 @@
         <v>170</v>
       </c>
       <c r="P212" t="n">
-        <v>600</v>
+        <v>650</v>
       </c>
       <c r="Q212" t="n">
-        <v>1350</v>
+        <v>1358</v>
       </c>
       <c r="R212"/>
       <c r="S212"/>
@@ -56109,7 +56299,7 @@
         <v>24</v>
       </c>
       <c r="V212" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="W212"/>
       <c r="X212"/>
@@ -56209,7 +56399,7 @@
       <c r="CZ212"/>
       <c r="DA212"/>
       <c r="DB212" t="n">
-        <v>3.66</v>
+        <v>2.66</v>
       </c>
       <c r="DC212" t="n">
         <v>-0.19764</v>
@@ -56353,10 +56543,10 @@
         <v>183</v>
       </c>
       <c r="P213" t="n">
-        <v>400</v>
+        <v>640</v>
       </c>
       <c r="Q213" t="n">
-        <v>1427</v>
+        <v>1448</v>
       </c>
       <c r="R213"/>
       <c r="S213"/>
@@ -56377,19 +56567,45 @@
       <c r="AB213"/>
       <c r="AC213"/>
       <c r="AD213"/>
-      <c r="AE213"/>
-      <c r="AF213"/>
-      <c r="AG213"/>
-      <c r="AH213"/>
-      <c r="AI213"/>
-      <c r="AJ213"/>
-      <c r="AK213"/>
-      <c r="AL213"/>
-      <c r="AM213"/>
-      <c r="AN213"/>
-      <c r="AO213"/>
-      <c r="AP213"/>
-      <c r="AQ213"/>
+      <c r="AE213" t="n">
+        <v>0.170586159355792</v>
+      </c>
+      <c r="AF213" t="n">
+        <v>1.37822466400964</v>
+      </c>
+      <c r="AG213" t="n">
+        <v>0.00214453867981628</v>
+      </c>
+      <c r="AH213" t="n">
+        <v>2.36476</v>
+      </c>
+      <c r="AI213" t="n">
+        <v>-0.763</v>
+      </c>
+      <c r="AJ213" t="n">
+        <v>-0.02285</v>
+      </c>
+      <c r="AK213" t="n">
+        <v>0.000074049</v>
+      </c>
+      <c r="AL213" t="n">
+        <v>-0.01018</v>
+      </c>
+      <c r="AM213" t="n">
+        <v>-0.27004</v>
+      </c>
+      <c r="AN213" t="n">
+        <v>1.09636482208082</v>
+      </c>
+      <c r="AO213" t="n">
+        <v>0.538</v>
+      </c>
+      <c r="AP213" t="n">
+        <v>0.667239487171173</v>
+      </c>
+      <c r="AQ213" t="n">
+        <v>0.817502081394196</v>
+      </c>
       <c r="AR213" t="n">
         <v>2.5</v>
       </c>
@@ -56811,10 +57027,10 @@
         <v>170</v>
       </c>
       <c r="P215" t="n">
-        <v>100</v>
+        <v>295</v>
       </c>
       <c r="Q215" t="n">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="R215"/>
       <c r="S215"/>
@@ -56869,7 +57085,7 @@
       <c r="BF215"/>
       <c r="BG215"/>
       <c r="BH215" t="n">
-        <v>2750</v>
+        <v>2747.25274725275</v>
       </c>
       <c r="BI215"/>
       <c r="BJ215"/>
@@ -56931,7 +57147,9 @@
       <c r="DF215" t="n">
         <v>25.26</v>
       </c>
-      <c r="DG215"/>
+      <c r="DG215" t="n">
+        <v>0.66</v>
+      </c>
       <c r="DH215" t="n">
         <v>-1.53691</v>
       </c>
@@ -57282,7 +57500,7 @@
         <v>790</v>
       </c>
       <c r="Q217" t="n">
-        <v>1263</v>
+        <v>1267</v>
       </c>
       <c r="R217" t="n">
         <v>182</v>
@@ -57417,7 +57635,7 @@
         <v>75.2475247524753</v>
       </c>
       <c r="DB217" t="n">
-        <v>0.0002464</v>
+        <v>0.65</v>
       </c>
       <c r="DC217" t="n">
         <v>-2.65</v>
@@ -57431,7 +57649,9 @@
       <c r="DF217" t="n">
         <v>18.6732186732187</v>
       </c>
-      <c r="DG217"/>
+      <c r="DG217" t="n">
+        <v>4.12</v>
+      </c>
       <c r="DH217" t="n">
         <v>-0.68</v>
       </c>
@@ -58029,10 +58249,10 @@
         <v>190</v>
       </c>
       <c r="P220" t="n">
-        <v>820</v>
+        <v>1110</v>
       </c>
       <c r="Q220" t="n">
-        <v>2780</v>
+        <v>2500</v>
       </c>
       <c r="R220" t="n">
         <v>100</v>
@@ -58042,10 +58262,10 @@
         <v>1676.4</v>
       </c>
       <c r="U220" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="V220" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="W220"/>
       <c r="X220"/>
@@ -58095,7 +58315,7 @@
       <c r="BF220"/>
       <c r="BG220"/>
       <c r="BH220" t="n">
-        <v>11054.10367</v>
+        <v>47619.0476190476</v>
       </c>
       <c r="BI220"/>
       <c r="BJ220" t="n">
@@ -58157,7 +58377,7 @@
       <c r="CZ220"/>
       <c r="DA220"/>
       <c r="DB220" t="n">
-        <v>1.64</v>
+        <v>3.39595</v>
       </c>
       <c r="DC220" t="n">
         <v>-2.32</v>
@@ -58553,10 +58773,10 @@
         <v>170</v>
       </c>
       <c r="P222" t="n">
-        <v>3000</v>
+        <v>650</v>
       </c>
       <c r="Q222" t="n">
-        <v>4226</v>
+        <v>2171</v>
       </c>
       <c r="R222" t="n">
         <v>79.58885</v>
@@ -58565,8 +58785,12 @@
       <c r="T222" t="n">
         <v>9136.8</v>
       </c>
-      <c r="U222"/>
-      <c r="V222"/>
+      <c r="U222" t="n">
+        <v>32</v>
+      </c>
+      <c r="V222" t="n">
+        <v>114</v>
+      </c>
       <c r="W222"/>
       <c r="X222"/>
       <c r="Y222"/>
@@ -58615,7 +58839,7 @@
       <c r="BF222"/>
       <c r="BG222"/>
       <c r="BH222" t="n">
-        <v>6000</v>
+        <v>5999.988000024</v>
       </c>
       <c r="BI222"/>
       <c r="BJ222" t="n">
@@ -58683,19 +58907,23 @@
       <c r="CZ222"/>
       <c r="DA222"/>
       <c r="DB222" t="n">
-        <v>0.11</v>
+        <v>2.64</v>
       </c>
       <c r="DC222" t="n">
         <v>-0.19</v>
       </c>
       <c r="DD222" t="n">
-        <v>-3.2</v>
-      </c>
-      <c r="DE222"/>
+        <v>-1.09</v>
+      </c>
+      <c r="DE222" t="n">
+        <v>-2.6</v>
+      </c>
       <c r="DF222" t="n">
-        <v>25.2491694352159</v>
-      </c>
-      <c r="DG222"/>
+        <v>31.5352697095436</v>
+      </c>
+      <c r="DG222" t="n">
+        <v>0.17</v>
+      </c>
       <c r="DH222" t="n">
         <v>-0.26</v>
       </c>
@@ -58843,10 +59071,10 @@
         <v>183</v>
       </c>
       <c r="P223" t="n">
-        <v>47.5</v>
+        <v>20</v>
       </c>
       <c r="Q223" t="n">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="R223"/>
       <c r="S223"/>
@@ -59103,10 +59331,10 @@
         <v>190</v>
       </c>
       <c r="P224" t="n">
-        <v>600</v>
+        <v>30</v>
       </c>
       <c r="Q224" t="n">
-        <v>600</v>
+        <v>537</v>
       </c>
       <c r="R224"/>
       <c r="S224"/>
@@ -59310,7 +59538,7 @@
         <v>100</v>
       </c>
       <c r="Q225" t="n">
-        <v>341</v>
+        <v>350</v>
       </c>
       <c r="R225"/>
       <c r="S225"/>
@@ -59581,10 +59809,10 @@
         <v>190</v>
       </c>
       <c r="P226" t="n">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="Q226" t="n">
-        <v>1314</v>
+        <v>1334</v>
       </c>
       <c r="R226"/>
       <c r="S226"/>
@@ -59921,7 +60149,7 @@
         <v>120.634920634921</v>
       </c>
       <c r="DB227" t="n">
-        <v>8.92857142857143</v>
+        <v>1.19</v>
       </c>
       <c r="DC227" t="n">
         <v>-1.34</v>

</xml_diff>